<commit_message>
WIP: report layout, tests, working-example data, and generated docs
Snapshot of in-progress work carried in the tree alongside the wordcloud
and report-styling changes: layout/section tweaks, booleplot/histogram/
treemap adjustments, test updates, refreshed working-example DGFs, and
regenerated man/ pages.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working-example/DGF-V2.xlsx
+++ b/working-example/DGF-V2.xlsx
@@ -103,7 +103,7 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "17,455"  ,  "PER" :  "(69.8%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,378"  ,  "PER" :  "(5.5%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "AMERICAN LEGION"  ,  "PER" :  "(2%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "AMERICAN LEGION"  ,  "PER" :  "(2.3%)"  }
 ]</t>
   </si>
   <si>
@@ -243,9 +243,9 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "10,990"  ,  "PER" :  "(44%)"  }, 
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "10,990"  ,  "PER" :  "(44.0%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "13,392"  ,  "PER" :  "(53.6%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "TREASURER"  ,  "PER" :  "(0%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "TREASURER"  ,  "PER" :  "(0.3%)"  }
 ]</t>
   </si>
   <si>
@@ -387,7 +387,7 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "18,785"  ,  "PER" :  "(75.1%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,378"  ,  "PER" :  "(5.5%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "9717 ELK GROVE FLORIN RD STE B"  ,  "PER" :  "(0%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "9717 ELK GROVE FLORIN RD STE B"  ,  "PER" :  "(0.1%)"  }
 ]</t>
   </si>
   <si>
@@ -529,7 +529,7 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "5,986"  ,  "PER" :  "(23.9%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,378"  ,  "PER" :  "(5.5%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "WASHINGTON"  ,  "PER" :  "(1%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "WASHINGTON"  ,  "PER" :  "(1.3%)"  }
 ]</t>
   </si>
   <si>
@@ -676,7 +676,7 @@
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "24,794"  ,  "PER" :  "(99.2%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "010100593"  ,  "PER" :  "(0%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "010100593"  ,  "PER" :  "(0.0%)"  }
 ]</t>
   </si>
   <si>
@@ -845,7 +845,7 @@
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "23"  ,  "PER" :  "(0.1%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "6"  ,  "PER" :  "(26%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "6"  ,  "PER" :  "(25.6%)"  }
 ]</t>
   </si>
   <si>
@@ -858,7 +858,24 @@
   {  "Value" :  "7"  ,  "Frequency" :  3571  }, 
   {  "Value" :  "5"  ,  "Frequency" :  3449  }, 
   {  "Value" :  "8"  ,  "Frequency" :  1479  }, 
-  {  "Value" :  "19"  ,  "Frequency" :  1459  }
+  {  "Value" :  "19"  ,  "Frequency" :  1459  }, 
+  {  "Value" :  "9"  ,  "Frequency" :  1033  }, 
+  {  "Value" :  "12"  ,  "Frequency" :  642  }, 
+  {  "Value" :  "13"  ,  "Frequency" :  561  }, 
+  {  "Value" :  "2"  ,  "Frequency" :  545  }, 
+  {  "Value" :  "10"  ,  "Frequency" :  466  }, 
+  {  "Value" :  "14"  ,  "Frequency" :  311  }, 
+  {  "Value" :  "25"  ,  "Frequency" :  88  }, 
+  {  "Value" :  "15"  ,  "Frequency" :  32  }, 
+  {  "Value" :  "17"  ,  "Frequency" :  22  }, 
+  {  "Value" :  "23"  ,  "Frequency" :  6  }, 
+  {  "Value" :  "11"  ,  "Frequency" :  2  }, 
+  {  "Value" :  "26"  ,  "Frequency" :  2  }, 
+  {  "Value" :  "16"  ,  "Frequency" :  1  }, 
+  {  "Value" :  "18"  ,  "Frequency" :  1  }, 
+  {  "Value" :  "24"  ,  "Frequency" :  1  }, 
+  {  "Value" :  "27"  ,  "Frequency" :  1  }, 
+  {  "Value" :  "29"  ,  "Frequency" :  1  }
 ]</t>
   </si>
   <si>
@@ -1133,7 +1150,7 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "230"  ,  "PER" :  "(0.9%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,887"  ,  "PER" :  "(7.5%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(23%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(23.2%)"  }
 ]</t>
   </si>
   <si>
@@ -1146,7 +1163,51 @@
   {  "Value" :  "200"  ,  "Frequency" :  1648  }, 
   {  "Value" :  "907"  ,  "Frequency" :  1212  }, 
   {  "Value" :  "36"  ,  "Frequency" :  1054  }, 
-  {  "Value" :  "279"  ,  "Frequency" :  998  }
+  {  "Value" :  "279"  ,  "Frequency" :  998  }, 
+  {  "Value" :  "205"  ,  "Frequency" :  949  }, 
+  {  "Value" :  "319"  ,  "Frequency" :  547  }, 
+  {  "Value" :  "318"  ,  "Frequency" :  467  }, 
+  {  "Value" :  "59"  ,  "Frequency" :  467  }, 
+  {  "Value" :  "407"  ,  "Frequency" :  401  }, 
+  {  "Value" :  "520"  ,  "Frequency" :  401  }, 
+  {  "Value" :  "900"  ,  "Frequency" :  323  }, 
+  {  "Value" :  "265"  ,  "Frequency" :  322  }, 
+  {  "Value" :  "264"  ,  "Frequency" :  301  }, 
+  {  "Value" :  "280"  ,  "Frequency" :  293  }, 
+  {  "Value" :  "260"  ,  "Frequency" :  276  }, 
+  {  "Value" :  "250"  ,  "Frequency" :  203  }, 
+  {  "Value" :  "999"  ,  "Frequency" :  200  }, 
+  {  "Value" :  "920"  ,  "Frequency" :  187  }, 
+  {  "Value" :  "30"  ,  "Frequency" :  179  }, 
+  {  "Value" :  "912"  ,  "Frequency" :  163  }, 
+  {  "Value" :  "261"  ,  "Frequency" :  162  }, 
+  {  "Value" :  "230"  ,  "Frequency" :  145  }, 
+  {  "Value" :  "65"  ,  "Frequency" :  143  }, 
+  {  "Value" :  "998"  ,  "Frequency" :  140  }, 
+  {  "Value" :  "229"  ,  "Frequency" :  137  }, 
+  {  "Value" :  "317"  ,  "Frequency" :  137  }, 
+  {  "Value" :  "403"  ,  "Frequency" :  136  }, 
+  {  "Value" :  "201"  ,  "Frequency" :  136  }, 
+  {  "Value" :  "908"  ,  "Frequency" :  125  }, 
+  {  "Value" :  "288"  ,  "Frequency" :  121  }, 
+  {  "Value" :  "911"  ,  "Frequency" :  120  }, 
+  {  "Value" :  "399"  ,  "Frequency" :  117  }, 
+  {  "Value" :  "286"  ,  "Frequency" :  115  }, 
+  {  "Value" :  "161"  ,  "Frequency" :  112  }, 
+  {  "Value" :  "922"  ,  "Frequency" :  97  }, 
+  {  "Value" :  "281"  ,  "Frequency" :  93  }, 
+  {  "Value" :  "350"  ,  "Frequency" :  91  }, 
+  {  "Value" :  "123"  ,  "Frequency" :  85  }, 
+  {  "Value" :  "287"  ,  "Frequency" :  78  }, 
+  {  "Value" :  "382"  ,  "Frequency" :  73  }, 
+  {  "Value" :  "401"  ,  "Frequency" :  69  }, 
+  {  "Value" :  "921"  ,  "Frequency" :  67  }, 
+  {  "Value" :  "34"  ,  "Frequency" :  60  }, 
+  {  "Value" :  "119"  ,  "Frequency" :  59  }, 
+  {  "Value" :  "408"  ,  "Frequency" :  58  }, 
+  {  "Value" :  "602"  ,  "Frequency" :  57  }, 
+  {  "Value" :  "251"  ,  "Frequency" :  56  }, 
+  {  "Value" :  "262"  ,  "Frequency" :  55  }
 ]</t>
   </si>
   <si>
@@ -1199,8 +1260,8 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "12"  ,  "PER" :  "(0%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "PU"  ,  "PER" :  "(37%)"  }
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "12"  ,  "PER" :  "(0.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "PU"  ,  "PER" :  "(36.5%)"  }
 ]</t>
   </si>
   <si>
@@ -1213,7 +1274,13 @@
   {  "Value" :  "MU"  ,  "Frequency" :  2480  }, 
   {  "Value" :  "ED"  ,  "Frequency" :  1528  }, 
   {  "Value" :  "UN"  ,  "Frequency" :  1524  }, 
-  {  "Value" :  "HE"  ,  "Frequency" :  994  }
+  {  "Value" :  "HE"  ,  "Frequency" :  994  }, 
+  {  "Value" :  "AR"  ,  "Frequency" :  615  }, 
+  {  "Value" :  "EN"  ,  "Frequency" :  508  }, 
+  {  "Value" :  "IN"  ,  "Frequency" :  101  }, 
+  {  "Value" :  "EH"  ,  "Frequency" :  79  }, 
+  {  "Value" :  "RE"  ,  "Frequency" :  64  }, 
+  {  "Value" :  "BH"  ,  "Frequency" :  24  }
 ]</t>
   </si>
   <si>
@@ -1279,8 +1346,8 @@
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "27"  ,  "PER" :  "(0.1%)"  }, 
-  {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,497"  ,  "PER" :  "(6%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "S"  ,  "PER" :  "(23%)"  }
+  {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,497"  ,  "PER" :  "(6.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "S"  ,  "PER" :  "(23.3%)"  }
 ]</t>
   </si>
   <si>
@@ -1293,7 +1360,27 @@
   {  "Value" :  "W"  ,  "Frequency" :  2835  }, 
   {  "Value" :  "Y"  ,  "Frequency" :  2480  }, 
   {  "Value" :  "J"  ,  "Frequency" :  1961  }, 
-  {  "Value" :  "B"  ,  "Frequency" :  1552  }
+  {  "Value" :  "B"  ,  "Frequency" :  1552  }, 
+  {  "Value" :  "M"  ,  "Frequency" :  876  }, 
+  {  "Value" :  "L"  ,  "Frequency" :  669  }, 
+  {  "Value" :  "A"  ,  "Frequency" :  615  }, 
+  {  "Value" :  "K"  ,  "Frequency" :  590  }, 
+  {  "Value" :  "E"  ,  "Frequency" :  574  }, 
+  {  "Value" :  "I"  ,  "Frequency" :  557  }, 
+  {  "Value" :  "G"  ,  "Frequency" :  382  }, 
+  {  "Value" :  "C"  ,  "Frequency" :  338  }, 
+  {  "Value" :  "P"  ,  "Frequency" :  210  }, 
+  {  "Value" :  "D"  ,  "Frequency" :  170  }, 
+  {  "Value" :  "U"  ,  "Frequency" :  166  }, 
+  {  "Value" :  "R"  ,  "Frequency" :  164  }, 
+  {  "Value" :  "T"  ,  "Frequency" :  142  }, 
+  {  "Value" :  "F"  ,  "Frequency" :  103  }, 
+  {  "Value" :  "Q"  ,  "Frequency" :  101  }, 
+  {  "Value" :  "O"  ,  "Frequency" :  74  }, 
+  {  "Value" :  "X"  ,  "Frequency" :  64  }, 
+  {  "Value" :  "Z"  ,  "Frequency" :  27  }, 
+  {  "Value" :  "H"  ,  "Frequency" :  14  }, 
+  {  "Value" :  "V"  ,  "Frequency" :  4  }
 ]</t>
   </si>
   <si>
@@ -1987,8 +2074,8 @@
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "654"  ,  "PER" :  "(2.6%)"  }, 
-  {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,497"  ,  "PER" :  "(6%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "S41"  ,  "PER" :  "(8%)"  }
+  {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,497"  ,  "PER" :  "(6.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "S41"  ,  "PER" :  "(7.8%)"  }
 ]</t>
   </si>
   <si>
@@ -2001,7 +2088,51 @@
   {  "Value" :  "W30"  ,  "Frequency" :  1582  }, 
   {  "Value" :  "S80"  ,  "Frequency" :  1515  }, 
   {  "Value" :  "N50"  ,  "Frequency" :  1088  }, 
-  {  "Value" :  "M24"  ,  "Frequency" :  810  }
+  {  "Value" :  "M24"  ,  "Frequency" :  810  }, 
+  {  "Value" :  "B83"  ,  "Frequency" :  771  }, 
+  {  "Value" :  "W80"  ,  "Frequency" :  681  }, 
+  {  "Value" :  "N60"  ,  "Frequency" :  600  }, 
+  {  "Value" :  "Y42"  ,  "Frequency" :  514  }, 
+  {  "Value" :  "Y50"  ,  "Frequency" :  484  }, 
+  {  "Value" :  "Y41"  ,  "Frequency" :  453  }, 
+  {  "Value" :  "K28"  ,  "Frequency" :  374  }, 
+  {  "Value" :  "S20"  ,  "Frequency" :  371  }, 
+  {  "Value" :  "Y43"  ,  "Frequency" :  355  }, 
+  {  "Value" :  "S47"  ,  "Frequency" :  347  }, 
+  {  "Value" :  "B03"  ,  "Frequency" :  346  }, 
+  {  "Value" :  "L50"  ,  "Frequency" :  328  }, 
+  {  "Value" :  "W61"  ,  "Frequency" :  270  }, 
+  {  "Value" :  "N61"  ,  "Frequency" :  269  }, 
+  {  "Value" :  "Y40"  ,  "Frequency" :  265  }, 
+  {  "Value" :  "S03"  ,  "Frequency" :  236  }, 
+  {  "Value" :  "Y20"  ,  "Frequency" :  236  }, 
+  {  "Value" :  "S30"  ,  "Frequency" :  214  }, 
+  {  "Value" :  "S01"  ,  "Frequency" :  201  }, 
+  {  "Value" :  "S40"  ,  "Frequency" :  185  }, 
+  {  "Value" :  "G90"  ,  "Frequency" :  173  }, 
+  {  "Value" :  "I03"  ,  "Frequency" :  172  }, 
+  {  "Value" :  "I0360"  ,  "Frequency" :  166  }, 
+  {  "Value" :  "N52"  ,  "Frequency" :  146  }, 
+  {  "Value" :  "S99"  ,  "Frequency" :  142  }, 
+  {  "Value" :  "A23"  ,  "Frequency" :  138  }, 
+  {  "Value" :  "S22"  ,  "Frequency" :  133  }, 
+  {  "Value" :  "N67"  ,  "Frequency" :  129  }, 
+  {  "Value" :  "N6A"  ,  "Frequency" :  124  }, 
+  {  "Value" :  "E11"  ,  "Frequency" :  100  }, 
+  {  "Value" :  "N68"  ,  "Frequency" :  98  }, 
+  {  "Value" :  "K20"  ,  "Frequency" :  93  }, 
+  {  "Value" :  "N69"  ,  "Frequency" :  92  }, 
+  {  "Value" :  "L99"  ,  "Frequency" :  89  }, 
+  {  "Value" :  "S46"  ,  "Frequency" :  89  }, 
+  {  "Value" :  "N32"  ,  "Frequency" :  78  }, 
+  {  "Value" :  "U42"  ,  "Frequency" :  77  }, 
+  {  "Value" :  "S21"  ,  "Frequency" :  74  }, 
+  {  "Value" :  "W20"  ,  "Frequency" :  72  }, 
+  {  "Value" :  "T20"  ,  "Frequency" :  70  }, 
+  {  "Value" :  "J22"  ,  "Frequency" :  68  }, 
+  {  "Value" :  "C32"  ,  "Frequency" :  65  }, 
+  {  "Value" :  "S81"  ,  "Frequency" :  64  }, 
+  {  "Value" :  "E03"  ,  "Frequency" :  64  }
 ]</t>
   </si>
   <si>
@@ -2057,7 +2188,7 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "16"  ,  "PER" :  "(0.1%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,378"  ,  "PER" :  "(5.5%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "BEST"  ,  "PER" :  "(50%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "BEST"  ,  "PER" :  "(49.6%)"  }
 ]</t>
   </si>
   <si>
@@ -2070,7 +2201,16 @@
   {  "Value" :  "NEW"  ,  "Frequency" :  2621  }, 
   {  "Value" :  "IRS"  ,  "Frequency" :  2540  }, 
   {  "Value" :  "SOI"  ,  "Frequency" :  855  }, 
-  {  "Value" :  "ZZ"  ,  "Frequency" :  454  }
+  {  "Value" :  "ZZ"  ,  "Frequency" :  454  }, 
+  {  "Value" :  "SUB"  ,  "Frequency" :  306  }, 
+  {  "Value" :  "SUB2"  ,  "Frequency" :  140  }, 
+  {  "Value" :  "SUB3"  ,  "Frequency" :  86  }, 
+  {  "Value" :  "ACT1"  ,  "Frequency" :  84  }, 
+  {  "Value" :  "VER"  ,  "Frequency" :  48  }, 
+  {  "Value" :  "ntCO"  ,  "Frequency" :  46  }, 
+  {  "Value" :  "HIED"  ,  "Frequency" :  19  }, 
+  {  "Value" :  "END2"  ,  "Frequency" :  11  }, 
+  {  "Value" :  "thp"  ,  "Frequency" :  2  }
 ]</t>
   </si>
   <si>
@@ -2109,9 +2249,9 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "5"  ,  "PER" :  "(0%)"  }, 
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "5"  ,  "PER" :  "(0.0%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,887"  ,  "PER" :  "(7.5%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "2"  ,  "PER" :  "(74%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "2"  ,  "PER" :  "(74.0%)"  }
 ]</t>
   </si>
   <si>
@@ -2159,9 +2299,9 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "5"  ,  "PER" :  "(0%)"  }, 
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "5"  ,  "PER" :  "(0.0%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "24,961"  ,  "PER" :  "(99.8%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "T"  ,  "PER" :  "(0%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "T"  ,  "PER" :  "(0.1%)"  }
 ]</t>
   </si>
   <si>
@@ -2209,8 +2349,8 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "2"  ,  "PER" :  "(0%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "N"  ,  "PER" :  "(86%)"  }
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "2"  ,  "PER" :  "(0.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "N"  ,  "PER" :  "(86.2%)"  }
 ]</t>
   </si>
   <si>
@@ -2250,9 +2390,9 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "3"  ,  "PER" :  "(0%)"  }, 
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "3"  ,  "PER" :  "(0.0%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "2,361"  ,  "PER" :  "(9.4%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "IN"  ,  "PER" :  "(90%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "IN"  ,  "PER" :  "(90.4%)"  }
 ]</t>
   </si>
   <si>
@@ -2293,7 +2433,9 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "2,411"  ,  "PER" :  "(9.6%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "2,389"  ,  "PER" :  "(9.6%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "6,037"  ,  "PER" :  "(2%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "6,037"  ,  "PER" :  "(1.6%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "LOW"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "MED"  ,  "PER" :  ""  }
 ]</t>
   </si>
   <si>
@@ -2316,300 +2458,72 @@
   <si>
     <t xml:space="preserve">  { 
     "breaks"  :  [ 
-1000, 
-    2000, 
-    3000, 
-    4000, 
+0, 
     5000, 
-    6000, 
-    7000, 
-    8000, 
-    9000, 
     10000, 
-    11000, 
-    12000, 
-    13000, 
-    14000, 
     15000, 
-    16000, 
-    17000, 
-    18000, 
-    19000, 
     20000, 
-    21000, 
-    22000, 
-    23000, 
-    24000, 
     25000, 
-    26000, 
-    27000, 
-    28000, 
-    29000, 
     30000, 
-    31000, 
-    32000, 
-    33000, 
-    34000, 
     35000, 
-    36000, 
-    37000, 
-    38000, 
-    39000, 
     40000, 
-    41000, 
-    42000, 
-    43000, 
-    44000, 
     45000, 
-    46000, 
-    47000, 
-    48000, 
-    49000, 
     50000, 
-    51000, 
-    52000, 
-    53000, 
-    54000, 
     55000, 
-    56000, 
-    57000, 
-    58000, 
-    59000, 
     60000, 
-    61000, 
-    62000, 
-    63000, 
-    64000, 
     65000, 
-    66000, 
-    67000, 
-    68000, 
-    69000, 
     70000, 
-    71000, 
-    72000, 
-    73000
+    75000
 ], 
     "density"  :  [ 
-0.0136, 
-    0.0054, 
-    0, 
-    0.0116, 
-    0.0078, 
-    0.093, 
-    0, 
-    0.0172, 
-    0.0156, 
-    0.0039, 
-    0.013, 
-    0.0361, 
-    0.021, 
-    0, 
-    0.0043, 
-    0.005, 
-    0.0476, 
-    0.0309, 
-    0.0175, 
-    0.0122, 
-    0.0131, 
-    0.0127, 
-    0.0067, 
-    0.0197, 
-    0.0305, 
-    0.0349, 
-    0.0278, 
-    0.0097, 
-    0.0229, 
-    0.0063, 
-    0.0083, 
-    0.0052, 
-    0.0056, 
-    0.031, 
-    0.0053, 
-    0.0647, 
-    0.022, 
-    0.0053, 
-    0.0437, 
-    0.0106, 
-    0.0143, 
-    0.0535, 
-    0, 
-    0.0055, 
-    0.0107, 
-    0.005, 
-    0.0155, 
-    0.0598, 
-    0.0049, 
-    0.0042, 
-    0.0276, 
-    0, 
-    0.0245, 
-    0.0088, 
-    0.0206, 
-    0.0028, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
+0.0306, 
+    0.1335, 
+    0.0741, 
+    0.1053, 
+    0.0644, 
+    0.1258, 
+    0.0564, 
+    0.141, 
+    0.084, 
+    0.0959, 
+    0.065, 
+    0.0234, 
     0, 
     0, 
     0.0005
 ], 
     "y"  :  [ 
-307, 
-    123, 
-    0, 
-    262, 
-    177, 
-    2102, 
-    0, 
-    388, 
-    352, 
-    89, 
-    294, 
-    817, 
-    475, 
-    0, 
-    97, 
-    113, 
-    1077, 
-    699, 
-    395, 
-    275, 
-    297, 
-    286, 
-    152, 
-    445, 
-    690, 
-    789, 
-    628, 
-    220, 
-    518, 
-    142, 
-    187, 
-    117, 
-    127, 
-    701, 
-    120, 
-    1463, 
-    497, 
-    120, 
-    988, 
-    240, 
-    324, 
-    1210, 
-    0, 
-    125, 
-    243, 
-    114, 
-    350, 
-    1352, 
-    110, 
-    95, 
-    623, 
-    0, 
-    553, 
-    199, 
-    466, 
-    63, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
+692, 
+    3019, 
+    1675, 
+    2381, 
+    1455, 
+    2845, 
+    1274, 
+    3188, 
+    1899, 
+    2169, 
+    1470, 
+    529, 
     0, 
     0, 
     12
 ], 
     "mids"  :  [ 
-1500, 
-    2500, 
-    3500, 
-    4500, 
-    5500, 
-    6500, 
+2500, 
     7500, 
-    8500, 
-    9500, 
-    10500, 
-    11500, 
     12500, 
-    13500, 
-    14500, 
-    15500, 
-    16500, 
     17500, 
-    18500, 
-    19500, 
-    20500, 
-    21500, 
     22500, 
-    23500, 
-    24500, 
-    25500, 
-    26500, 
     27500, 
-    28500, 
-    29500, 
-    30500, 
-    31500, 
     32500, 
-    33500, 
-    34500, 
-    35500, 
-    36500, 
     37500, 
-    38500, 
-    39500, 
-    40500, 
-    41500, 
     42500, 
-    43500, 
-    44500, 
-    45500, 
-    46500, 
     47500, 
-    48500, 
-    49500, 
-    50500, 
-    51500, 
     52500, 
-    53500, 
-    54500, 
-    55500, 
-    56500, 
     57500, 
-    58500, 
-    59500, 
-    60500, 
-    61500, 
     62500, 
-    63500, 
-    64500, 
-    65500, 
-    66500, 
     67500, 
-    68500, 
-    69500, 
-    70500, 
-    71500, 
     72500
 ], 
     "mean"  :  [ 
@@ -2647,7 +2561,9 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "14,265"  ,  "PER" :  "(57.1%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "3,110"  ,  "PER" :  "(12.4%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "NA"  ,  "PER" :  "(0%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "11,001,010,700"  ,  "PER" :  "(0.3%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "LOW"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "MED"  ,  "PER" :  ""  }
 ]</t>
   </si>
   <si>
@@ -2670,457 +2586,129 @@
   <si>
     <t xml:space="preserve">  { 
     "breaks"  :  [ 
-1000000000, 
-    1500000000, 
+0, 
     2000000000, 
-    2500000000, 
-    3000000000, 
-    3500000000, 
     4000000000, 
-    4500000000, 
-    5000000000, 
-    5500000000, 
     6000000000, 
-    6500000000, 
-    7000000000, 
-    7500000000, 
     8000000000, 
-    8500000000, 
-    9000000000, 
-    9500000000, 
     10000000000, 
-    10500000000, 
-    11000000000, 
-    11500000000, 
     12000000000, 
-    12500000000, 
-    13000000000, 
-    13500000000, 
     14000000000, 
-    14500000000, 
-    15000000000, 
-    15500000000, 
     16000000000, 
-    16500000000, 
-    17000000000, 
-    17500000000, 
     18000000000, 
-    18500000000, 
-    19000000000, 
-    19500000000, 
     20000000000, 
-    20500000000, 
-    21000000000, 
-    21500000000, 
     22000000000, 
-    22500000000, 
-    23000000000, 
-    23500000000, 
     24000000000, 
-    24500000000, 
-    25000000000, 
-    25500000000, 
     26000000000, 
-    26500000000, 
-    27000000000, 
-    27500000000, 
     28000000000, 
-    28500000000, 
-    29000000000, 
-    29500000000, 
     30000000000, 
-    30500000000, 
-    31000000000, 
-    31500000000, 
     32000000000, 
-    32500000000, 
-    33000000000, 
-    33500000000, 
     34000000000, 
-    34500000000, 
-    35000000000, 
-    35500000000, 
     36000000000, 
-    36500000000, 
-    37000000000, 
-    37500000000, 
     38000000000, 
-    38500000000, 
-    39000000000, 
-    39500000000, 
     40000000000, 
-    40500000000, 
-    41000000000, 
-    41500000000, 
     42000000000, 
-    42500000000, 
-    43000000000, 
-    43500000000, 
     44000000000, 
-    44500000000, 
-    45000000000, 
-    45500000000, 
     46000000000, 
-    46500000000, 
-    47000000000, 
-    47500000000, 
     48000000000, 
-    48500000000, 
-    49000000000, 
-    49500000000, 
     50000000000, 
-    50500000000, 
-    51000000000, 
-    51500000000, 
     52000000000, 
-    52500000000, 
-    53000000000, 
-    53500000000, 
     54000000000, 
-    54500000000, 
-    55000000000, 
-    55500000000, 
     56000000000, 
-    56500000000
+    58000000000
 ], 
     "density"  :  [ 
 0.0136, 
-    0, 
     0.0051, 
-    0, 
-    0, 
-    0, 
-    0.0105, 
-    0, 
-    0.0079, 
-    0, 
+    0.0184, 
     0.0912, 
-    0, 
-    0, 
-    0, 
-    0.0173, 
-    0, 
-    0.0159, 
-    0, 
-    0.004, 
-    0, 
-    0.0128, 
-    0, 
+    0.0332, 
+    0.0168, 
+    0.057, 
+    0.0037, 
+    0.0527, 
+    0.0489, 
+    0.0259, 
+    0.0195, 
+    0.0506, 
+    0.0631, 
+    0.0331, 
+    0.0148, 
+    0.0107, 
     0.036, 
-    0, 
-    0.0209, 
-    0, 
-    0, 
-    0, 
-    0.0037, 
-    0, 
-    0.0049, 
-    0, 
-    0.0478, 
-    0, 
-    0.031, 
-    0, 
-    0.0179, 
-    0, 
-    0.0124, 
-    0, 
-    0.0135, 
-    0, 
-    0.0128, 
-    0, 
-    0.0067, 
-    0, 
-    0.018, 
-    0.0018, 
-    0.0307, 
-    0, 
-    0.0352, 
-    0, 
-    0.0279, 
-    0, 
-    0.01, 
-    0, 
-    0.0208, 
-    0.0023, 
-    0.0063, 
-    0, 
-    0.0084, 
-    0, 
-    0.0048, 
-    0.0003, 
-    0.0057, 
-    0, 
-    0.0307, 
-    0, 
-    0.0053, 
-    0, 
-    0.0644, 
-    0, 
-    0.022, 
-    0, 
-    0.0053, 
-    0, 
-    0.0441, 
-    0, 
-    0.0106, 
-    0, 
-    0.0132, 
-    0, 
+    0.0863, 
+    0.0494, 
+    0.0237, 
     0.0545, 
-    0, 
-    0, 
-    0, 
-    0.0055, 
-    0, 
-    0.0106, 
-    0, 
-    0.0052, 
-    0, 
-    0.0158, 
-    0, 
-    0.0606, 
-    0.0002, 
-    0.0049, 
-    0, 
-    0.0042, 
-    0, 
-    0.0166, 
-    0.0111, 
-    0, 
-    0, 
+    0.0162, 
+    0.021, 
+    0.0657, 
+    0.0319, 
     0.0248, 
-    0, 
-    0.0087, 
-    0, 
-    0.0209, 
-    0, 
+    0.0296, 
     0.0029
 ], 
     "y"  :  [ 
 297, 
-    0, 
     111, 
-    0, 
-    0, 
-    0, 
-    229, 
-    0, 
-    173, 
-    0, 
+    402, 
     1996, 
-    0, 
-    0, 
-    0, 
-    379, 
-    0, 
-    348, 
-    0, 
-    87, 
-    0, 
-    280, 
-    0, 
+    727, 
+    367, 
+    1247, 
+    81, 
+    1153, 
+    1070, 
+    566, 
+    426, 
+    1107, 
+    1382, 
+    724, 
+    323, 
+    234, 
     789, 
-    0, 
-    458, 
-    0, 
-    0, 
-    0, 
-    81, 
-    0, 
-    107, 
-    0, 
-    1046, 
-    0, 
-    679, 
-    0, 
-    391, 
-    0, 
-    271, 
-    0, 
-    295, 
-    0, 
-    280, 
-    0, 
-    146, 
-    0, 
-    395, 
-    40, 
-    672, 
-    0, 
-    771, 
-    0, 
-    611, 
-    0, 
-    218, 
-    0, 
-    455, 
-    51, 
-    139, 
-    0, 
-    184, 
-    0, 
-    104, 
-    6, 
-    124, 
-    0, 
-    673, 
-    0, 
-    116, 
-    0, 
-    1409, 
-    0, 
-    481, 
-    0, 
-    117, 
-    0, 
-    965, 
-    0, 
-    231, 
-    0, 
-    288, 
-    0, 
+    1890, 
+    1082, 
+    519, 
     1194, 
-    0, 
-    0, 
-    0, 
-    121, 
-    0, 
-    233, 
-    0, 
-    114, 
-    0, 
-    345, 
-    0, 
-    1326, 
-    5, 
-    108, 
-    0, 
-    92, 
-    0, 
-    363, 
-    243, 
-    0, 
-    0, 
+    354, 
+    459, 
+    1439, 
+    698, 
     543, 
-    0, 
-    190, 
-    0, 
-    457, 
-    0, 
+    647, 
     63
 ], 
     "mids"  :  [ 
-1250000000, 
-    1750000000, 
-    2250000000, 
-    2750000000, 
-    3250000000, 
-    3750000000, 
-    4250000000, 
-    4750000000, 
-    5250000000, 
-    5750000000, 
-    6250000000, 
-    6750000000, 
-    7250000000, 
-    7750000000, 
-    8250000000, 
-    8750000000, 
-    9250000000, 
-    9750000000, 
-    10250000000, 
-    10750000000, 
-    11250000000, 
-    11750000000, 
-    12250000000, 
-    12750000000, 
-    13250000000, 
-    13750000000, 
-    14250000000, 
-    14750000000, 
-    15250000000, 
-    15750000000, 
-    16250000000, 
-    16750000000, 
-    17250000000, 
-    17750000000, 
-    18250000000, 
-    18750000000, 
-    19250000000, 
-    19750000000, 
-    20250000000, 
-    20750000000, 
-    21250000000, 
-    21750000000, 
-    22250000000, 
-    22750000000, 
-    23250000000, 
-    23750000000, 
-    24250000000, 
-    24750000000, 
-    25250000000, 
-    25750000000, 
-    26250000000, 
-    26750000000, 
-    27250000000, 
-    27750000000, 
-    28250000000, 
-    28750000000, 
-    29250000000, 
-    29750000000, 
-    30250000000, 
-    30750000000, 
-    31250000000, 
-    31750000000, 
-    32250000000, 
-    32750000000, 
-    33250000000, 
-    33750000000, 
-    34250000000, 
-    34750000000, 
-    35250000000, 
-    35750000000, 
-    36250000000, 
-    36750000000, 
-    37250000000, 
-    37750000000, 
-    38250000000, 
-    38750000000, 
-    39250000000, 
-    39750000000, 
-    40250000000, 
-    40750000000, 
-    41250000000, 
-    41750000000, 
-    42250000000, 
-    42750000000, 
-    43250000000, 
-    43750000000, 
-    44250000000, 
-    44750000000, 
-    45250000000, 
-    45750000000, 
-    46250000000, 
-    46750000000, 
-    47250000000, 
-    47750000000, 
-    48250000000, 
-    48750000000, 
-    49250000000, 
-    49750000000, 
-    50250000000, 
-    50750000000, 
-    51250000000, 
-    51750000000, 
-    52250000000, 
-    52750000000, 
-    53250000000, 
-    53750000000, 
-    54250000000, 
-    54750000000, 
-    55250000000, 
-    55750000000, 
-    56250000000
+1000000000, 
+    3000000000, 
+    5000000000, 
+    7000000000, 
+    9000000000, 
+    11000000000, 
+    13000000000, 
+    15000000000, 
+    17000000000, 
+    19000000000, 
+    21000000000, 
+    23000000000, 
+    25000000000, 
+    27000000000, 
+    29000000000, 
+    31000000000, 
+    33000000000, 
+    35000000000, 
+    37000000000, 
+    39000000000, 
+    41000000000, 
+    43000000000, 
+    45000000000, 
+    47000000000, 
+    49000000000, 
+    51000000000, 
+    53000000000, 
+    55000000000, 
+    57000000000
 ], 
     "mean"  :  [ 
 28488147052.6496
@@ -3210,7 +2798,7 @@
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "47"  ,  "PER" :  "(0.2%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "2019-12"  ,  "PER" :  "(40%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "2019-12"  ,  "PER" :  "(39.5%)"  }
 ]</t>
   </si>
   <si>
@@ -3223,7 +2811,48 @@
   {  "Value" :  "2019-06"  ,  "Frequency" :  2064  }, 
   {  "Value" :  "2017-12"  ,  "Frequency" :  1626  }, 
   {  "Value" :  "2020-06"  ,  "Frequency" :  1312  }, 
-  {  "Value" :  "2018-06"  ,  "Frequency" :  840  }
+  {  "Value" :  "2018-06"  ,  "Frequency" :  840  }, 
+  {  "Value" :  "2019-09"  ,  "Frequency" :  812  }, 
+  {  "Value" :  "2019-08"  ,  "Frequency" :  406  }, 
+  {  "Value" :  "2017-06"  ,  "Frequency" :  362  }, 
+  {  "Value" :  "2019-03"  ,  "Frequency" :  356  }, 
+  {  "Value" :  "2020-03"  ,  "Frequency" :  352  }, 
+  {  "Value" :  "2019-05"  ,  "Frequency" :  326  }, 
+  {  "Value" :  "2019-04"  ,  "Frequency" :  278  }, 
+  {  "Value" :  "2019-10"  ,  "Frequency" :  272  }, 
+  {  "Value" :  "2020-05"  ,  "Frequency" :  252  }, 
+  {  "Value" :  "2018-09"  ,  "Frequency" :  244  }, 
+  {  "Value" :  "2020-04"  ,  "Frequency" :  183  }, 
+  {  "Value" :  "2019-07"  ,  "Frequency" :  161  }, 
+  {  "Value" :  "2018-05"  ,  "Frequency" :  154  }, 
+  {  "Value" :  "2018-08"  ,  "Frequency" :  139  }, 
+  {  "Value" :  "2019-11"  ,  "Frequency" :  123  }, 
+  {  "Value" :  "2017-09"  ,  "Frequency" :  121  }, 
+  {  "Value" :  "2018-03"  ,  "Frequency" :  110  }, 
+  {  "Value" :  "2018-04"  ,  "Frequency" :  102  }, 
+  {  "Value" :  "2018-10"  ,  "Frequency" :  94  }, 
+  {  "Value" :  "2020-07"  ,  "Frequency" :  91  }, 
+  {  "Value" :  "2020-08"  ,  "Frequency" :  79  }, 
+  {  "Value" :  "2020-09"  ,  "Frequency" :  74  }, 
+  {  "Value" :  "2020-01"  ,  "Frequency" :  66  }, 
+  {  "Value" :  "2018-07"  ,  "Frequency" :  65  }, 
+  {  "Value" :  "2017-05"  ,  "Frequency" :  64  }, 
+  {  "Value" :  "2017-08"  ,  "Frequency" :  64  }, 
+  {  "Value" :  "2020-02"  ,  "Frequency" :  59  }, 
+  {  "Value" :  "2019-02"  ,  "Frequency" :  57  }, 
+  {  "Value" :  "2017-04"  ,  "Frequency" :  46  }, 
+  {  "Value" :  "2017-10"  ,  "Frequency" :  46  }, 
+  {  "Value" :  "2018-11"  ,  "Frequency" :  46  }, 
+  {  "Value" :  "2019-01"  ,  "Frequency" :  34  }, 
+  {  "Value" :  "2017-07"  ,  "Frequency" :  32  }, 
+  {  "Value" :  "2018-02"  ,  "Frequency" :  32  }, 
+  {  "Value" :  "2017-03"  ,  "Frequency" :  31  }, 
+  {  "Value" :  "2017-11"  ,  "Frequency" :  25  }, 
+  {  "Value" :  "2020-10"  ,  "Frequency" :  13  }, 
+  {  "Value" :  "2018-01"  ,  "Frequency" :  9  }, 
+  {  "Value" :  "2017-01"  ,  "Frequency" :  8  }, 
+  {  "Value" :  "2017-02"  ,  "Frequency" :  8  }, 
+  {  "Value" :  "2020-11"  ,  "Frequency" :  1  }
 ]</t>
   </si>
   <si>
@@ -3309,7 +2938,7 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "47"  ,  "PER" :  "(0.2%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "4,344"  ,  "PER" :  "(17.4%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "2018-12"  ,  "PER" :  "(37%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "2018-12"  ,  "PER" :  "(37.2%)"  }
 ]</t>
   </si>
   <si>
@@ -3322,7 +2951,47 @@
   {  "Value" :  "2018-06"  ,  "Frequency" :  1767  }, 
   {  "Value" :  "2019-06"  ,  "Frequency" :  1060  }, 
   {  "Value" :  "2018-09"  ,  "Frequency" :  744  }, 
-  {  "Value" :  "2017-06"  ,  "Frequency" :  539  }
+  {  "Value" :  "2017-06"  ,  "Frequency" :  539  }, 
+  {  "Value" :  "2016-12"  ,  "Frequency" :  478  }, 
+  {  "Value" :  "2018-08"  ,  "Frequency" :  370  }, 
+  {  "Value" :  "2018-03"  ,  "Frequency" :  321  }, 
+  {  "Value" :  "2019-03"  ,  "Frequency" :  319  }, 
+  {  "Value" :  "2018-05"  ,  "Frequency" :  265  }, 
+  {  "Value" :  "2018-10"  ,  "Frequency" :  255  }, 
+  {  "Value" :  "2018-04"  ,  "Frequency" :  246  }, 
+  {  "Value" :  "2019-05"  ,  "Frequency" :  206  }, 
+  {  "Value" :  "2017-09"  ,  "Frequency" :  195  }, 
+  {  "Value" :  "2016-06"  ,  "Frequency" :  164  }, 
+  {  "Value" :  "2019-04"  ,  "Frequency" :  162  }, 
+  {  "Value" :  "2018-07"  ,  "Frequency" :  123  }, 
+  {  "Value" :  "2018-11"  ,  "Frequency" :  122  }, 
+  {  "Value" :  "2017-08"  ,  "Frequency" :  101  }, 
+  {  "Value" :  "2017-05"  ,  "Frequency" :  90  }, 
+  {  "Value" :  "2017-10"  ,  "Frequency" :  88  }, 
+  {  "Value" :  "2017-04"  ,  "Frequency" :  64  }, 
+  {  "Value" :  "2019-01"  ,  "Frequency" :  61  }, 
+  {  "Value" :  "2019-07"  ,  "Frequency" :  58  }, 
+  {  "Value" :  "2017-03"  ,  "Frequency" :  51  }, 
+  {  "Value" :  "2019-02"  ,  "Frequency" :  49  }, 
+  {  "Value" :  "2018-02"  ,  "Frequency" :  46  }, 
+  {  "Value" :  "2019-08"  ,  "Frequency" :  44  }, 
+  {  "Value" :  "2019-09"  ,  "Frequency" :  42  }, 
+  {  "Value" :  "2017-11"  ,  "Frequency" :  41  }, 
+  {  "Value" :  "2017-07"  ,  "Frequency" :  39  }, 
+  {  "Value" :  "2016-05"  ,  "Frequency" :  36  }, 
+  {  "Value" :  "2016-09"  ,  "Frequency" :  34  }, 
+  {  "Value" :  "2018-01"  ,  "Frequency" :  29  }, 
+  {  "Value" :  "2016-04"  ,  "Frequency" :  27  }, 
+  {  "Value" :  "2016-08"  ,  "Frequency" :  23  }, 
+  {  "Value" :  "2017-02"  ,  "Frequency" :  22  }, 
+  {  "Value" :  "2016-03"  ,  "Frequency" :  18  }, 
+  {  "Value" :  "2016-07"  ,  "Frequency" :  16  }, 
+  {  "Value" :  "2016-10"  ,  "Frequency" :  13  }, 
+  {  "Value" :  "2016-11"  ,  "Frequency" :  9  }, 
+  {  "Value" :  "2019-10"  ,  "Frequency" :  7  }, 
+  {  "Value" :  "2016-01"  ,  "Frequency" :  5  }, 
+  {  "Value" :  "2016-02"  ,  "Frequency" :  4  }, 
+  {  "Value" :  "2017-01"  ,  "Frequency" :  3  }
 ]</t>
   </si>
   <si>
@@ -3356,8 +3025,8 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "12"  ,  "PER" :  "(0%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "2019-0"  ,  "PER" :  "(41%)"  }
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "12"  ,  "PER" :  "(0.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "2019-0"  ,  "PER" :  "(40.8%)"  }
 ]</t>
   </si>
   <si>
@@ -3473,8 +3142,8 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "12"  ,  "PER" :  "(0%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "12"  ,  "PER" :  "(60%)"  }
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "12"  ,  "PER" :  "(0.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "12"  ,  "PER" :  "(59.9%)"  }
 ]</t>
   </si>
   <si>
@@ -3487,7 +3156,13 @@
   {  "Value" :  "09"  ,  "Frequency" :  1251  }, 
   {  "Value" :  "03"  ,  "Frequency" :  849  }, 
   {  "Value" :  "05"  ,  "Frequency" :  796  }, 
-  {  "Value" :  "08"  ,  "Frequency" :  688  }
+  {  "Value" :  "08"  ,  "Frequency" :  688  }, 
+  {  "Value" :  "04"  ,  "Frequency" :  609  }, 
+  {  "Value" :  "10"  ,  "Frequency" :  425  }, 
+  {  "Value" :  "07"  ,  "Frequency" :  349  }, 
+  {  "Value" :  "11"  ,  "Frequency" :  195  }, 
+  {  "Value" :  "02"  ,  "Frequency" :  156  }, 
+  {  "Value" :  "01"  ,  "Frequency" :  117  }
 ]</t>
   </si>
   <si>
@@ -3523,7 +3198,9 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "23,817"  ,  "PER" :  "(95.3%)"  }, 
   {  "STAT" :  "Zero"  ,  "VAL" :  "413"  ,  "PER" :  "(1.7%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(2%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(1.7%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }
 ]</t>
   </si>
   <si>
@@ -3546,819 +3223,7 @@
   <si>
     <t xml:space="preserve">  { 
     "breaks"  :  [ 
--460000, 
-    -440000, 
-    -420000, 
-    -400000, 
-    -380000, 
-    -360000, 
-    -340000, 
-    -320000, 
-    -300000, 
-    -280000, 
-    -260000, 
-    -240000, 
-    -220000, 
-    -200000, 
-    -180000, 
-    -160000, 
-    -140000, 
-    -120000, 
-    -100000, 
-    -80000, 
-    -60000, 
-    -40000, 
-    -20000, 
-    0, 
-    20000, 
-    40000, 
-    60000, 
-    80000, 
-    100000, 
-    120000, 
-    140000, 
-    160000, 
-    180000, 
-    200000, 
-    220000, 
-    240000, 
-    260000, 
-    280000, 
-    300000, 
-    320000, 
-    340000, 
-    360000, 
-    380000, 
-    400000, 
-    420000, 
-    440000, 
-    460000, 
-    480000, 
-    500000, 
-    520000, 
-    540000, 
-    560000, 
-    580000, 
-    600000, 
-    620000, 
-    640000, 
-    660000, 
-    680000, 
-    700000, 
-    720000, 
-    740000, 
-    760000, 
-    780000, 
-    800000, 
-    820000, 
-    840000, 
-    860000, 
-    880000, 
-    900000, 
-    920000, 
-    940000, 
-    960000, 
-    980000, 
-    1000000, 
-    1020000, 
-    1040000
-], 
-    "density"  :  [ 
-0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0.0001, 
-    0.0001, 
-    0, 
-    0, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0004, 
-    0.0003, 
-    0.0006, 
-    0.0008, 
-    0.0236, 
-    0.1169, 
-    0.0951, 
-    0.1052, 
-    0.0901, 
-    0.0719, 
-    0.0577, 
-    0.0466, 
-    0.0405, 
-    0.0328, 
-    0.0295, 
-    0.0222, 
-    0.0216, 
-    0.0189, 
-    0.0175, 
-    0.0141, 
-    0.0151, 
-    0.0126, 
-    0.0108, 
-    0.0107, 
-    0.0094, 
-    0.0086, 
-    0.0079, 
-    0.009, 
-    0.0071, 
-    0.0062, 
-    0.0065, 
-    0.0062, 
-    0.0058, 
-    0.0043, 
-    0.0049, 
-    0.0052, 
-    0.0043, 
-    0.0043, 
-    0.0044, 
-    0.0039, 
-    0.0033, 
-    0.0035, 
-    0.0036, 
-    0.0033, 
-    0.0036, 
-    0.0029, 
-    0.0024, 
-    0.0027, 
-    0.0035, 
-    0.0032, 
-    0.0024, 
-    0.0016, 
-    0.0023, 
-    0.0018, 
-    0.0024, 
-    0.0022, 
-    0.001
-], 
-    "y"  :  [ 
-1, 
-    1, 
-    0, 
-    1, 
-    0, 
-    0, 
-    1, 
-    1, 
-    0, 
-    0, 
-    1, 
-    2, 
-    2, 
-    1, 
-    1, 
-    2, 
-    3, 
-    2, 
-    8, 
-    6, 
-    13, 
-    17, 
-    501, 
-    2481, 
-    2018, 
-    2233, 
-    1913, 
-    1525, 
-    1224, 
-    990, 
-    860, 
-    697, 
-    627, 
-    472, 
-    458, 
-    401, 
-    372, 
-    299, 
-    320, 
-    267, 
-    229, 
-    228, 
-    200, 
-    182, 
-    167, 
-    190, 
-    150, 
-    131, 
-    138, 
-    131, 
-    124, 
-    91, 
-    103, 
-    111, 
-    91, 
-    91, 
-    94, 
-    83, 
-    70, 
-    75, 
-    76, 
-    69, 
-    77, 
-    61, 
-    51, 
-    57, 
-    74, 
-    68, 
-    50, 
-    35, 
-    48, 
-    39, 
-    50, 
-    46, 
-    21
-], 
-    "mids"  :  [ 
--450000, 
-    -430000, 
-    -410000, 
-    -390000, 
-    -370000, 
-    -350000, 
-    -330000, 
-    -310000, 
-    -290000, 
-    -270000, 
-    -250000, 
-    -230000, 
-    -210000, 
-    -190000, 
-    -170000, 
-    -150000, 
-    -130000, 
-    -110000, 
-    -90000, 
-    -70000, 
-    -50000, 
-    -30000, 
-    -10000, 
-    10000, 
-    30000, 
-    50000, 
-    70000, 
-    90000, 
-    110000, 
-    130000, 
-    150000, 
-    170000, 
-    190000, 
-    210000, 
-    230000, 
-    250000, 
-    270000, 
-    290000, 
-    310000, 
-    330000, 
-    350000, 
-    370000, 
-    390000, 
-    410000, 
-    430000, 
-    450000, 
-    470000, 
-    490000, 
-    510000, 
-    530000, 
-    550000, 
-    570000, 
-    590000, 
-    610000, 
-    630000, 
-    650000, 
-    670000, 
-    690000, 
-    710000, 
-    730000, 
-    750000, 
-    770000, 
-    790000, 
-    810000, 
-    830000, 
-    850000, 
-    870000, 
-    890000, 
-    910000, 
-    930000, 
-    950000, 
-    970000, 
-    990000, 
-    1010000, 
-    1030000
-], 
-    "mean"  :  [ 
-3740777.062
-], 
-    "median"  :  [ 
-130545
-], 
-    "min"  :  [ 
--61467591
-], 
-    "max"  :  [ 
-4178522311
-]
-  }</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d2e4429d44416d4fd723ee541e73d2a3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F9_10_ASSET_TOT_BOY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total assets - beginning of year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34227234 ;; 
-17491720 ;; 
-101131 ;; 
-0 ;; 
-3011522</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 
-  {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "20,195"  ,  "PER" :  "(80.8%)"  }, 
-  {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,377"  ,  "PER" :  "(5.5%)"  }, 
-  {  "STAT" :  "Zero"  ,  "VAL" :  "3,011"  ,  "PER" :  "(12%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(12%)"  }
-]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 ;; 1 ;; 300 ;; 161 ;; 1593 ;; 10571 ;; 20855 ;; 21915 ;; 43506 ;; 49481 ;; 2 ;; 97 ;; 212 ;; 219 ;; 343 ;; 388 ;; 500 ;; 718 ;; 1000 ;; 1020 ;; 1222 ;; 1535 ;; 1547 ;; 1607 ;; 1642 ;; 2155 ;; 2745 ;; 3068 ;; 3073 ;; 3087 ;; 3708 ;; 4412 ;; 4414 ;; 4612 ;; 5251 ;; 5501 ;; 5619 ;; 5761 ;; 6141 ;; 6267 ;; 6812 ;; 6865 ;; 7575 ;; 8302 ;; 8451 ;; 8528 ;; 8853 ;; 9083 ;; 9110 ;; 9369 ;; 9527 ;; 9937</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 
-  {  "STAT" :  "Minimum"  ,  "VAL" :  "-69,049"  }, 
-  {  "STAT" :  "Q - 05"  ,  "VAL" :  "0"  }, 
-  {  "STAT" :  "Q - 25"  ,  "VAL" :  "31,558.5"  }, 
-  {  "STAT" :  "Median"  ,  "VAL" :  "169,734"  }, 
-  {  "STAT" :  "Mean"  ,  "VAL" :  "11,116,959"  }, 
-  {  "STAT" :  "Q - 75"  ,  "VAL" :  "729,844.5"  }, 
-  {  "STAT" :  "Q - 95"  ,  "VAL" :  "13,488,117"  }, 
-  {  "STAT" :  "Maximum"  ,  "VAL" :  "11,226,543,829"  }, 
-  {  "STAT" :  "Skew"  ,  "VAL" :  "41.82"  }, 
-  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "2,117.75"  }
-]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  { 
-    "breaks"  :  [ 
--80000, 
-    -60000, 
-    -40000, 
-    -20000, 
-    0, 
-    20000, 
-    40000, 
-    60000, 
-    80000, 
-    100000, 
-    120000, 
-    140000, 
-    160000, 
-    180000, 
-    200000, 
-    220000, 
-    240000, 
-    260000, 
-    280000, 
-    300000, 
-    320000, 
-    340000, 
-    360000, 
-    380000, 
-    400000, 
-    420000, 
-    440000, 
-    460000, 
-    480000, 
-    500000, 
-    520000, 
-    540000, 
-    560000, 
-    580000, 
-    600000, 
-    620000, 
-    640000, 
-    660000, 
-    680000, 
-    700000, 
-    720000, 
-    740000, 
-    760000, 
-    780000, 
-    800000, 
-    820000, 
-    840000, 
-    860000, 
-    880000, 
-    900000, 
-    920000, 
-    940000, 
-    960000, 
-    980000, 
-    1000000, 
-    1020000, 
-    1040000, 
-    1060000, 
-    1080000, 
-    1100000, 
-    1120000, 
-    1140000, 
-    1160000, 
-    1180000, 
-    1200000, 
-    1220000, 
-    1240000, 
-    1260000, 
-    1280000, 
-    1300000, 
-    1320000, 
-    1340000, 
-    1360000, 
-    1380000, 
-    1400000, 
-    1420000, 
-    1440000, 
-    1460000, 
-    1480000, 
-    1500000, 
-    1520000, 
-    1540000, 
-    1560000, 
-    1580000, 
-    1600000, 
-    1620000, 
-    1640000, 
-    1660000, 
-    1680000, 
-    1700000, 
-    1720000, 
-    1740000, 
-    1760000, 
-    1780000
-], 
-    "density"  :  [ 
-0, 
-    0, 
-    0, 
-    0.151, 
-    0.0976, 
-    0.077, 
-    0.0617, 
-    0.052, 
-    0.0414, 
-    0.0352, 
-    0.0315, 
-    0.0283, 
-    0.0269, 
-    0.0232, 
-    0.0211, 
-    0.0199, 
-    0.0177, 
-    0.016, 
-    0.0137, 
-    0.0145, 
-    0.0123, 
-    0.0128, 
-    0.0108, 
-    0.0114, 
-    0.0103, 
-    0.009, 
-    0.0088, 
-    0.0087, 
-    0.0077, 
-    0.0072, 
-    0.0065, 
-    0.0057, 
-    0.006, 
-    0.006, 
-    0.0056, 
-    0.0052, 
-    0.0056, 
-    0.005, 
-    0.0041, 
-    0.0047, 
-    0.0041, 
-    0.0035, 
-    0.0044, 
-    0.0042, 
-    0.0037, 
-    0.0045, 
-    0.0034, 
-    0.0033, 
-    0.0035, 
-    0.0036, 
-    0.0028, 
-    0.003, 
-    0.0026, 
-    0.0028, 
-    0.0029, 
-    0.003, 
-    0.003, 
-    0.0029, 
-    0.002, 
-    0.0022, 
-    0.0029, 
-    0.002, 
-    0.0018, 
-    0.0023, 
-    0.0013, 
-    0.0022, 
-    0.0018, 
-    0.0021, 
-    0.0014, 
-    0.0014, 
-    0.0019, 
-    0.002, 
-    0.0016, 
-    0.0014, 
-    0.0018, 
-    0.0016, 
-    0.0012, 
-    0.0012, 
-    0.0013, 
-    0.0016, 
-    0.0016, 
-    0.0014, 
-    0.0009, 
-    0.0014, 
-    0.0011, 
-    0.0018, 
-    0.0007, 
-    0.0014, 
-    0.0013, 
-    0.0014, 
-    0.0013, 
-    0.0012, 
-    0.0009
-], 
-    "y"  :  [ 
-1, 
-    0, 
-    0, 
-    3027, 
-    1957, 
-    1544, 
-    1237, 
-    1042, 
-    830, 
-    706, 
-    631, 
-    567, 
-    539, 
-    465, 
-    422, 
-    399, 
-    354, 
-    320, 
-    275, 
-    290, 
-    246, 
-    256, 
-    217, 
-    228, 
-    207, 
-    180, 
-    176, 
-    174, 
-    154, 
-    145, 
-    131, 
-    115, 
-    121, 
-    121, 
-    112, 
-    105, 
-    113, 
-    100, 
-    82, 
-    95, 
-    82, 
-    71, 
-    88, 
-    84, 
-    75, 
-    90, 
-    69, 
-    67, 
-    71, 
-    73, 
-    56, 
-    60, 
-    52, 
-    57, 
-    59, 
-    60, 
-    60, 
-    58, 
-    40, 
-    45, 
-    58, 
-    41, 
-    37, 
-    47, 
-    26, 
-    45, 
-    36, 
-    42, 
-    29, 
-    29, 
-    39, 
-    41, 
-    32, 
-    29, 
-    36, 
-    32, 
-    25, 
-    24, 
-    26, 
-    32, 
-    32, 
-    29, 
-    18, 
-    29, 
-    23, 
-    37, 
-    15, 
-    29, 
-    26, 
-    29, 
-    27, 
-    25, 
-    19
-], 
-    "mids"  :  [ 
--70000, 
-    -50000, 
-    -30000, 
-    -10000, 
-    10000, 
-    30000, 
-    50000, 
-    70000, 
-    90000, 
-    110000, 
-    130000, 
-    150000, 
-    170000, 
-    190000, 
-    210000, 
-    230000, 
-    250000, 
-    270000, 
-    290000, 
-    310000, 
-    330000, 
-    350000, 
-    370000, 
-    390000, 
-    410000, 
-    430000, 
-    450000, 
-    470000, 
-    490000, 
-    510000, 
-    530000, 
-    550000, 
-    570000, 
-    590000, 
-    610000, 
-    630000, 
-    650000, 
-    670000, 
-    690000, 
-    710000, 
-    730000, 
-    750000, 
-    770000, 
-    790000, 
-    810000, 
-    830000, 
-    850000, 
-    870000, 
-    890000, 
-    910000, 
-    930000, 
-    950000, 
-    970000, 
-    990000, 
-    1010000, 
-    1030000, 
-    1050000, 
-    1070000, 
-    1090000, 
-    1110000, 
-    1130000, 
-    1150000, 
-    1170000, 
-    1190000, 
-    1210000, 
-    1230000, 
-    1250000, 
-    1270000, 
-    1290000, 
-    1310000, 
-    1330000, 
-    1350000, 
-    1370000, 
-    1390000, 
-    1410000, 
-    1430000, 
-    1450000, 
-    1470000, 
-    1490000, 
-    1510000, 
-    1530000, 
-    1550000, 
-    1570000, 
-    1590000, 
-    1610000, 
-    1630000, 
-    1650000, 
-    1670000, 
-    1690000, 
-    1710000, 
-    1730000, 
-    1750000, 
-    1770000
-], 
-    "mean"  :  [ 
-11116958.5761
-], 
-    "median"  :  [ 
-169734
-], 
-    "min"  :  [ 
--69049
-], 
-    "max"  :  [ 
-11226543829
-]
-  }</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e70794cebd95ead0ac4363dfeb80cf83</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F9_10_ASSET_TOT_EOY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total assets - end of year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40131275 ;; 
-20157050 ;; 
-92924 ;; 
-19430176 ;; 
-2856785</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 
-  {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "24,122"  ,  "PER" :  "(96.5%)"  }, 
-  {  "STAT" :  "Zero"  ,  "VAL" :  "110"  ,  "PER" :  "(0.4%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "1"  ,  "PER" :  "(1%)"  }
-]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 ;; 0 ;; 100 ;; 1000 ;; 15000 ;; 21 ;; 480 ;; 529 ;; 680 ;; 1257 ;; 1374 ;; 1932 ;; 2000 ;; 2076 ;; 2280 ;; 2680 ;; 2965 ;; 3000 ;; 10000 ;; 24731 ;; 24753 ;; 37977 ;; 40760 ;; 25 ;; 30 ;; 39 ;; 90 ;; 99 ;; 140 ;; 149 ;; 200 ;; 212 ;; 230 ;; 248 ;; 249 ;; 281 ;; 314 ;; 340 ;; 415 ;; 459 ;; 478 ;; 627 ;; 628 ;; 663 ;; 912 ;; 957 ;; 997 ;; 1107 ;; 1158 ;; 1203 ;; 1353 ;; 1383 ;; 1389 ;; 1500 ;; 163</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 
-  {  "STAT" :  "Minimum"  ,  "VAL" :  "-1,119,570"  }, 
-  {  "STAT" :  "Q - 05"  ,  "VAL" :  "4,421.45"  }, 
-  {  "STAT" :  "Q - 25"  ,  "VAL" :  "55,668.25"  }, 
-  {  "STAT" :  "Median"  ,  "VAL" :  "212,649"  }, 
-  {  "STAT" :  "Mean"  ,  "VAL" :  "13,755,826"  }, 
-  {  "STAT" :  "Q - 75"  ,  "VAL" :  "837,286"  }, 
-  {  "STAT" :  "Q - 95"  ,  "VAL" :  "14,639,755"  }, 
-  {  "STAT" :  "Maximum"  ,  "VAL" :  "38,468,314,242"  }, 
-  {  "STAT" :  "Skew"  ,  "VAL" :  "85.67"  }, 
-  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "9,676.68"  }
-]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  { 
-    "breaks"  :  [ 
--850000, 
-    -800000, 
-    -750000, 
-    -700000, 
-    -650000, 
-    -600000, 
-    -550000, 
-    -500000, 
+-500000, 
     -450000, 
     -400000, 
     -350000, 
@@ -4389,157 +3254,76 @@
     900000, 
     950000, 
     1000000, 
-    1050000, 
-    1100000, 
-    1150000, 
-    1200000, 
-    1250000, 
-    1300000, 
-    1350000, 
-    1400000, 
-    1450000, 
-    1500000, 
-    1550000, 
-    1600000, 
-    1650000, 
-    1700000, 
-    1750000, 
-    1800000, 
-    1850000, 
-    1900000, 
-    1950000, 
-    2000000, 
-    2050000
+    1050000
 ], 
     "density"  :  [ 
 0, 
     0, 
     0, 
+    0.0001, 
     0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0.0065, 
-    0.2678, 
-    0.1381, 
-    0.0919, 
-    0.0713, 
-    0.0526, 
-    0.0442, 
-    0.0378, 
-    0.0297, 
-    0.025, 
-    0.0242, 
-    0.0183, 
-    0.0173, 
-    0.0148, 
-    0.0141, 
-    0.0126, 
-    0.0113, 
-    0.01, 
+    0.0002, 
+    0.0001, 
+    0.0003, 
+    0.0009, 
+    0.0248, 
+    0.2622, 
+    0.217, 
+    0.1239, 
+    0.0833, 
+    0.0536, 
+    0.0407, 
+    0.0331, 
+    0.0255, 
+    0.0212, 
+    0.0174, 
+    0.0161, 
+    0.0115, 
+    0.0119, 
+    0.0102, 
+    0.0085, 
     0.0088, 
-    0.0085, 
-    0.0083, 
+    0.0067, 
     0.0079, 
-    0.0067, 
-    0.0063, 
-    0.0063, 
-    0.006, 
-    0.0044, 
-    0.0048, 
-    0.0048, 
-    0.0046, 
-    0.0042, 
-    0.0039, 
-    0.0039, 
-    0.003, 
-    0.0033, 
-    0.0027, 
-    0.0037, 
-    0.0021, 
-    0.0026, 
-    0.003, 
-    0.0018, 
-    0.0006
+    0.0051, 
+    0.0053, 
+    0.0032
 ], 
     "y"  :  [ 
 1, 
+    1, 
+    1, 
+    2, 
     0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    1, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    138, 
-    5677, 
-    2927, 
-    1947, 
-    1511, 
-    1115, 
-    937, 
-    802, 
-    630, 
-    530, 
-    513, 
-    388, 
-    366, 
-    314, 
-    298, 
-    267, 
-    240, 
-    212, 
-    187, 
+    5, 
+    3, 
+    6, 
+    19, 
+    526, 
+    5565, 
+    4605, 
+    2630, 
+    1768, 
+    1138, 
+    864, 
+    702, 
+    542, 
+    450, 
+    370, 
+    342, 
+    245, 
+    253, 
+    217, 
     181, 
-    175, 
+    186, 
+    143, 
     168, 
-    142, 
-    134, 
-    133, 
-    128, 
-    93, 
-    101, 
-    102, 
-    98, 
-    90, 
-    82, 
-    82, 
-    64, 
-    70, 
-    58, 
-    79, 
-    45, 
-    56, 
-    64, 
-    38, 
-    12
+    109, 
+    113, 
+    67
 ], 
     "mids"  :  [ 
--825000, 
-    -775000, 
-    -725000, 
-    -675000, 
-    -625000, 
-    -575000, 
-    -525000, 
-    -475000, 
+-475000, 
     -425000, 
     -375000, 
     -325000, 
@@ -4569,27 +3353,340 @@
     875000, 
     925000, 
     975000, 
-    1025000, 
-    1075000, 
-    1125000, 
-    1175000, 
-    1225000, 
-    1275000, 
-    1325000, 
-    1375000, 
-    1425000, 
-    1475000, 
-    1525000, 
-    1575000, 
-    1625000, 
-    1675000, 
-    1725000, 
-    1775000, 
-    1825000, 
-    1875000, 
-    1925000, 
-    1975000, 
-    2025000
+    1025000
+], 
+    "mean"  :  [ 
+3740777.062
+], 
+    "median"  :  [ 
+130545
+], 
+    "min"  :  [ 
+-61467591
+], 
+    "max"  :  [ 
+4178522311
+]
+  }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d2e4429d44416d4fd723ee541e73d2a3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F9_10_ASSET_TOT_BOY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total assets - beginning of year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34227234 ;; 
+17491720 ;; 
+101131 ;; 
+0 ;; 
+3011522</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[ 
+  {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "20,195"  ,  "PER" :  "(80.8%)"  }, 
+  {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,377"  ,  "PER" :  "(5.5%)"  }, 
+  {  "STAT" :  "Zero"  ,  "VAL" :  "3,011"  ,  "PER" :  "(12.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(12.0%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 ;; 1 ;; 300 ;; 161 ;; 1593 ;; 10571 ;; 20855 ;; 21915 ;; 43506 ;; 49481 ;; 2 ;; 97 ;; 212 ;; 219 ;; 343 ;; 388 ;; 500 ;; 718 ;; 1000 ;; 1020 ;; 1222 ;; 1535 ;; 1547 ;; 1607 ;; 1642 ;; 2155 ;; 2745 ;; 3068 ;; 3073 ;; 3087 ;; 3708 ;; 4412 ;; 4414 ;; 4612 ;; 5251 ;; 5501 ;; 5619 ;; 5761 ;; 6141 ;; 6267 ;; 6812 ;; 6865 ;; 7575 ;; 8302 ;; 8451 ;; 8528 ;; 8853 ;; 9083 ;; 9110 ;; 9369 ;; 9527 ;; 9937</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[ 
+  {  "STAT" :  "Minimum"  ,  "VAL" :  "-69,049"  }, 
+  {  "STAT" :  "Q - 05"  ,  "VAL" :  "0"  }, 
+  {  "STAT" :  "Q - 25"  ,  "VAL" :  "31,558.5"  }, 
+  {  "STAT" :  "Median"  ,  "VAL" :  "169,734"  }, 
+  {  "STAT" :  "Mean"  ,  "VAL" :  "11,116,959"  }, 
+  {  "STAT" :  "Q - 75"  ,  "VAL" :  "729,844.5"  }, 
+  {  "STAT" :  "Q - 95"  ,  "VAL" :  "13,488,117"  }, 
+  {  "STAT" :  "Maximum"  ,  "VAL" :  "11,226,543,829"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "41.82"  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "2,117.75"  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  { 
+    "breaks"  :  [ 
+-100000, 
+    0, 
+    100000, 
+    200000, 
+    300000, 
+    400000, 
+    500000, 
+    600000, 
+    700000, 
+    800000, 
+    900000, 
+    1000000, 
+    1100000, 
+    1200000, 
+    1300000, 
+    1400000, 
+    1500000, 
+    1600000, 
+    1700000, 
+    1800000
+], 
+    "density"  :  [ 
+0.1511, 
+    0.3298, 
+    0.1451, 
+    0.0883, 
+    0.0617, 
+    0.0444, 
+    0.0316, 
+    0.0255, 
+    0.021, 
+    0.0186, 
+    0.0149, 
+    0.0138, 
+    0.0114, 
+    0.0089, 
+    0.0085, 
+    0.0071, 
+    0.007, 
+    0.0065, 
+    0.005
+], 
+    "y"  :  [ 
+3028, 
+    6610, 
+    2908, 
+    1770, 
+    1237, 
+    891, 
+    633, 
+    512, 
+    420, 
+    372, 
+    298, 
+    277, 
+    228, 
+    178, 
+    170, 
+    143, 
+    140, 
+    130, 
+    100
+], 
+    "mids"  :  [ 
+-50000, 
+    50000, 
+    150000, 
+    250000, 
+    350000, 
+    450000, 
+    550000, 
+    650000, 
+    750000, 
+    850000, 
+    950000, 
+    1050000, 
+    1150000, 
+    1250000, 
+    1350000, 
+    1450000, 
+    1550000, 
+    1650000, 
+    1750000
+], 
+    "mean"  :  [ 
+11116958.5761
+], 
+    "median"  :  [ 
+169734
+], 
+    "min"  :  [ 
+-69049
+], 
+    "max"  :  [ 
+11226543829
+]
+  }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e70794cebd95ead0ac4363dfeb80cf83</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F9_10_ASSET_TOT_EOY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total assets - end of year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40131275 ;; 
+20157050 ;; 
+92924 ;; 
+19430176 ;; 
+2856785</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[ 
+  {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "24,122"  ,  "PER" :  "(96.5%)"  }, 
+  {  "STAT" :  "Zero"  ,  "VAL" :  "110"  ,  "PER" :  "(0.4%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "1"  ,  "PER" :  "(1.1%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 ;; 0 ;; 100 ;; 1000 ;; 15000 ;; 21 ;; 480 ;; 529 ;; 680 ;; 1257 ;; 1374 ;; 1932 ;; 2000 ;; 2076 ;; 2280 ;; 2680 ;; 2965 ;; 3000 ;; 10000 ;; 24731 ;; 24753 ;; 37977 ;; 40760 ;; 25 ;; 30 ;; 39 ;; 90 ;; 99 ;; 140 ;; 149 ;; 200 ;; 212 ;; 230 ;; 248 ;; 249 ;; 281 ;; 314 ;; 340 ;; 415 ;; 459 ;; 478 ;; 627 ;; 628 ;; 663 ;; 912 ;; 957 ;; 997 ;; 1107 ;; 1158 ;; 1203 ;; 1353 ;; 1383 ;; 1389 ;; 1500 ;; 163</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[ 
+  {  "STAT" :  "Minimum"  ,  "VAL" :  "-1,119,570"  }, 
+  {  "STAT" :  "Q - 05"  ,  "VAL" :  "4,421.45"  }, 
+  {  "STAT" :  "Q - 25"  ,  "VAL" :  "55,668.25"  }, 
+  {  "STAT" :  "Median"  ,  "VAL" :  "212,649"  }, 
+  {  "STAT" :  "Mean"  ,  "VAL" :  "13,755,826"  }, 
+  {  "STAT" :  "Q - 75"  ,  "VAL" :  "837,286"  }, 
+  {  "STAT" :  "Q - 95"  ,  "VAL" :  "14,639,755"  }, 
+  {  "STAT" :  "Maximum"  ,  "VAL" :  "38,468,314,242"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "85.67"  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "9,676.68"  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  { 
+    "breaks"  :  [ 
+-900000, 
+    -800000, 
+    -700000, 
+    -600000, 
+    -500000, 
+    -400000, 
+    -300000, 
+    -200000, 
+    -100000, 
+    0, 
+    100000, 
+    200000, 
+    300000, 
+    400000, 
+    500000, 
+    600000, 
+    700000, 
+    800000, 
+    900000, 
+    1000000, 
+    1100000, 
+    1200000, 
+    1300000, 
+    1400000, 
+    1500000, 
+    1600000, 
+    1700000, 
+    1800000, 
+    1900000, 
+    2000000, 
+    2100000
+], 
+    "density"  :  [ 
+0, 
+    0, 
+    0, 
+    0, 
+    0, 
+    0, 
+    0, 
+    0, 
+    0.0065, 
+    0.4059, 
+    0.1631, 
+    0.0968, 
+    0.0676, 
+    0.0492, 
+    0.0356, 
+    0.0289, 
+    0.0239, 
+    0.0188, 
+    0.0168, 
+    0.0146, 
+    0.0126, 
+    0.0104, 
+    0.0096, 
+    0.0089, 
+    0.0077, 
+    0.0063, 
+    0.0065, 
+    0.0048, 
+    0.0048, 
+    0.0006
+], 
+    "y"  :  [ 
+1, 
+    0, 
+    0, 
+    0, 
+    1, 
+    0, 
+    0, 
+    0, 
+    138, 
+    8604, 
+    3458, 
+    2052, 
+    1432, 
+    1043, 
+    754, 
+    612, 
+    507, 
+    399, 
+    356, 
+    310, 
+    267, 
+    221, 
+    203, 
+    188, 
+    164, 
+    134, 
+    137, 
+    101, 
+    102, 
+    12
+], 
+    "mids"  :  [ 
+-850000, 
+    -750000, 
+    -650000, 
+    -550000, 
+    -450000, 
+    -350000, 
+    -250000, 
+    -150000, 
+    -50000, 
+    50000, 
+    150000, 
+    250000, 
+    350000, 
+    450000, 
+    550000, 
+    650000, 
+    750000, 
+    850000, 
+    950000, 
+    1050000, 
+    1150000, 
+    1250000, 
+    1350000, 
+    1450000, 
+    1550000, 
+    1650000, 
+    1750000, 
+    1850000, 
+    1950000, 
+    2050000
 ], 
     "mean"  :  [ 
 13755826.3585
@@ -4627,7 +3724,9 @@
   {  "STAT" :  "Distinct"  ,  "VAL" :  "20,145"  ,  "PER" :  "(80.6%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "4,344"  ,  "PER" :  "(17.4%)"  }, 
   {  "STAT" :  "Zero"  ,  "VAL" :  "203"  ,  "PER" :  "(0.8%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(1%)"  }
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(0.8%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }
 ]</t>
   </si>
   <si>
@@ -4650,553 +3749,125 @@
   <si>
     <t xml:space="preserve">  { 
     "breaks"  :  [ 
--960000, 
-    -940000, 
-    -920000, 
+-1000000, 
     -900000, 
-    -880000, 
-    -860000, 
-    -840000, 
-    -820000, 
     -800000, 
-    -780000, 
-    -760000, 
-    -740000, 
-    -720000, 
     -700000, 
-    -680000, 
-    -660000, 
-    -640000, 
-    -620000, 
     -600000, 
-    -580000, 
-    -560000, 
-    -540000, 
-    -520000, 
     -500000, 
-    -480000, 
-    -460000, 
-    -440000, 
-    -420000, 
     -400000, 
-    -380000, 
-    -360000, 
-    -340000, 
-    -320000, 
     -300000, 
-    -280000, 
-    -260000, 
-    -240000, 
-    -220000, 
     -200000, 
-    -180000, 
-    -160000, 
-    -140000, 
-    -120000, 
     -100000, 
-    -80000, 
-    -60000, 
-    -40000, 
-    -20000, 
     0, 
-    20000, 
-    40000, 
-    60000, 
-    80000, 
     100000, 
-    120000, 
-    140000, 
-    160000, 
-    180000, 
     200000, 
-    220000, 
-    240000, 
-    260000, 
-    280000, 
     300000, 
-    320000, 
-    340000, 
-    360000, 
-    380000, 
     400000, 
-    420000, 
-    440000, 
-    460000, 
-    480000, 
     500000, 
-    520000, 
-    540000, 
-    560000, 
-    580000, 
     600000, 
-    620000, 
-    640000, 
-    660000, 
-    680000, 
     700000, 
-    720000, 
-    740000, 
-    760000, 
-    780000, 
     800000, 
-    820000, 
-    840000, 
-    860000, 
-    880000, 
     900000, 
-    920000, 
-    940000, 
-    960000, 
-    980000, 
     1000000, 
-    1020000, 
-    1040000, 
-    1060000, 
-    1080000, 
     1100000, 
-    1120000, 
-    1140000, 
-    1160000, 
-    1180000, 
     1200000, 
-    1220000, 
-    1240000, 
-    1260000, 
-    1280000, 
     1300000, 
-    1320000, 
-    1340000, 
-    1360000, 
-    1380000, 
     1400000, 
-    1420000, 
-    1440000, 
-    1460000, 
-    1480000, 
     1500000, 
-    1520000, 
-    1540000, 
-    1560000, 
-    1580000, 
     1600000, 
-    1620000, 
-    1640000, 
-    1660000, 
-    1680000, 
     1700000, 
-    1720000, 
-    1740000
+    1800000
 ], 
     "density"  :  [ 
 0.0001, 
-    0, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0002, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0001, 
-    0.0003, 
-    0.0003, 
-    0.0002, 
-    0.0005, 
-    0.0002, 
-    0.0001, 
-    0.0002, 
-    0.0002, 
-    0.0002, 
-    0.0002, 
-    0.0003, 
-    0.0002, 
-    0.0002, 
     0.0003, 
     0.0005, 
-    0.0005, 
-    0.0007, 
-    0.0005, 
-    0.0006, 
-    0.0005, 
-    0.0007, 
-    0.0005, 
-    0.0016, 
-    0.0011, 
-    0.0014, 
+    0.0003, 
+    0.001, 
+    0.0012, 
+    0.0012, 
     0.0026, 
-    0.004, 
-    0.0215, 
-    0.109, 
-    0.0918, 
-    0.0729, 
-    0.061, 
-    0.0474, 
-    0.0424, 
-    0.0373, 
-    0.0324, 
-    0.0299, 
+    0.0039, 
+    0.0306, 
+    0.3822, 
+    0.1684, 
+    0.102, 
+    0.0682, 
+    0.0496, 
+    0.0347, 
     0.0263, 
-    0.025, 
-    0.0234, 
-    0.0202, 
-    0.0179, 
-    0.0154, 
-    0.0164, 
-    0.0131, 
-    0.0144, 
-    0.0124, 
-    0.0119, 
-    0.0101, 
-    0.0103, 
-    0.0107, 
-    0.0095, 
-    0.0089, 
-    0.0089, 
-    0.0074, 
-    0.0058, 
-    0.006, 
-    0.0066, 
-    0.005, 
-    0.0056, 
-    0.006, 
-    0.0052, 
-    0.0043, 
-    0.0054, 
-    0.0056, 
-    0.0045, 
-    0.0044, 
-    0.0043, 
-    0.0039, 
-    0.0043, 
-    0.0041, 
-    0.004, 
-    0.0042, 
-    0.003, 
-    0.0029, 
-    0.0034, 
-    0.0028, 
-    0.0027, 
-    0.0025, 
-    0.0034, 
-    0.0024, 
-    0.0036, 
-    0.0019, 
-    0.0024, 
-    0.0025, 
-    0.0022, 
-    0.0019, 
-    0.0015, 
-    0.0021, 
-    0.0018, 
-    0.0022, 
-    0.0022, 
-    0.0016, 
-    0.0018, 
-    0.0018, 
-    0.0023, 
-    0.0017, 
-    0.0013, 
-    0.0018, 
-    0.0018, 
-    0.0018, 
-    0.0014, 
-    0.0014, 
-    0.0014, 
-    0.0021, 
-    0.0014, 
-    0.0015, 
-    0.0014, 
-    0.0014, 
-    0.0012, 
-    0.0015, 
-    0.0014, 
-    0.0015, 
-    0.0016, 
-    0.0001
+    0.0242, 
+    0.0205, 
+    0.0148, 
+    0.0139, 
+    0.0105, 
+    0.0098, 
+    0.009, 
+    0.0082, 
+    0.0077, 
+    0.007, 
+    0.0017
 ], 
     "y"  :  [ 
-1, 
-    0, 
-    1, 
-    1, 
-    1, 
-    1, 
-    1, 
-    2, 
-    3, 
-    1, 
-    2, 
-    2, 
-    1, 
-    1, 
-    1, 
-    0, 
-    2, 
-    2, 
-    1, 
-    2, 
-    5, 
-    5, 
-    4, 
-    8, 
-    4, 
-    2, 
-    4, 
-    3, 
-    3, 
-    4, 
+2, 
     6, 
-    4, 
-    4, 
+    9, 
     6, 
-    8, 
-    9, 
-    13, 
-    9, 
-    10, 
-    9, 
-    12, 
-    9, 
-    28, 
-    19, 
-    25, 
+    17, 
+    21, 
+    21, 
     45, 
-    70, 
-    377, 
-    1912, 
-    1610, 
-    1278, 
-    1070, 
-    832, 
-    744, 
-    655, 
-    569, 
-    524, 
+    68, 
+    536, 
+    6702, 
+    2953, 
+    1788, 
+    1196, 
+    869, 
+    608, 
     461, 
-    439, 
-    410, 
-    355, 
-    314, 
-    270, 
-    287, 
-    230, 
-    253, 
-    217, 
-    209, 
-    178, 
-    181, 
-    187, 
-    167, 
-    156, 
-    156, 
-    130, 
-    101, 
-    105, 
-    116, 
-    88, 
-    99, 
-    106, 
-    92, 
-    76, 
-    94, 
-    99, 
-    79, 
-    78, 
-    75, 
-    68, 
-    75, 
-    72, 
-    71, 
-    73, 
-    52, 
-    50, 
-    60, 
-    49, 
-    48, 
-    44, 
-    60, 
-    42, 
-    64, 
-    33, 
-    42, 
-    43, 
-    38, 
-    34, 
-    27, 
-    36, 
-    31, 
-    38, 
-    38, 
-    28, 
-    31, 
-    32, 
-    41, 
-    30, 
-    23, 
-    32, 
-    32, 
-    31, 
-    24, 
-    25, 
-    24, 
-    37, 
-    24, 
-    26, 
-    24, 
-    24, 
-    21, 
-    27, 
-    25, 
-    26, 
-    28, 
-    1
+    425, 
+    359, 
+    259, 
+    243, 
+    184, 
+    171, 
+    157, 
+    144, 
+    135, 
+    123, 
+    29
 ], 
     "mids"  :  [ 
 -950000, 
-    -930000, 
-    -910000, 
-    -890000, 
-    -870000, 
     -850000, 
-    -830000, 
-    -810000, 
-    -790000, 
-    -770000, 
     -750000, 
-    -730000, 
-    -710000, 
-    -690000, 
-    -670000, 
     -650000, 
-    -630000, 
-    -610000, 
-    -590000, 
-    -570000, 
     -550000, 
-    -530000, 
-    -510000, 
-    -490000, 
-    -470000, 
     -450000, 
-    -430000, 
-    -410000, 
-    -390000, 
-    -370000, 
     -350000, 
-    -330000, 
-    -310000, 
-    -290000, 
-    -270000, 
     -250000, 
-    -230000, 
-    -210000, 
-    -190000, 
-    -170000, 
     -150000, 
-    -130000, 
-    -110000, 
-    -90000, 
-    -70000, 
     -50000, 
-    -30000, 
-    -10000, 
-    10000, 
-    30000, 
     50000, 
-    70000, 
-    90000, 
-    110000, 
-    130000, 
     150000, 
-    170000, 
-    190000, 
-    210000, 
-    230000, 
     250000, 
-    270000, 
-    290000, 
-    310000, 
-    330000, 
     350000, 
-    370000, 
-    390000, 
-    410000, 
-    430000, 
     450000, 
-    470000, 
-    490000, 
-    510000, 
-    530000, 
     550000, 
-    570000, 
-    590000, 
-    610000, 
-    630000, 
     650000, 
-    670000, 
-    690000, 
-    710000, 
-    730000, 
     750000, 
-    770000, 
-    790000, 
-    810000, 
-    830000, 
     850000, 
-    870000, 
-    890000, 
-    910000, 
-    930000, 
     950000, 
-    970000, 
-    990000, 
-    1010000, 
-    1030000, 
     1050000, 
-    1070000, 
-    1090000, 
-    1110000, 
-    1130000, 
     1150000, 
-    1170000, 
-    1190000, 
-    1210000, 
-    1230000, 
     1250000, 
-    1270000, 
-    1290000, 
-    1310000, 
-    1330000, 
     1350000, 
-    1370000, 
-    1390000, 
-    1410000, 
-    1430000, 
     1450000, 
-    1470000, 
-    1490000, 
-    1510000, 
-    1530000, 
     1550000, 
-    1570000, 
-    1590000, 
-    1610000, 
-    1630000, 
     1650000, 
-    1670000, 
-    1690000, 
-    1710000, 
-    1730000
+    1750000
 ], 
     "mean"  :  [ 
 4921982.0918
@@ -5231,9 +3902,11 @@
   <si>
     <t xml:space="preserve">[ 
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
-  {  "STAT" :  "Distinct"  ,  "VAL" :  "23,740"  ,  "PER" :  "(95%)"  }, 
-  {  "STAT" :  "Zero"  ,  "VAL" :  "489"  ,  "PER" :  "(2%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(2%)"  }
+  {  "STAT" :  "Distinct"  ,  "VAL" :  "23,740"  ,  "PER" :  "(95.0%)"  }, 
+  {  "STAT" :  "Zero"  ,  "VAL" :  "489"  ,  "PER" :  "(2.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(2.0%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }
 ]</t>
   </si>
   <si>
@@ -5256,405 +3929,97 @@
   <si>
     <t xml:space="preserve">  { 
     "breaks"  :  [ 
--20000, 
-    -10000, 
+-50000, 
     0, 
-    10000, 
-    20000, 
-    30000, 
-    40000, 
     50000, 
-    60000, 
-    70000, 
-    80000, 
-    90000, 
     100000, 
-    110000, 
-    120000, 
-    130000, 
-    140000, 
     150000, 
-    160000, 
-    170000, 
-    180000, 
-    190000, 
     200000, 
-    210000, 
-    220000, 
-    230000, 
-    240000, 
     250000, 
-    260000, 
-    270000, 
-    280000, 
-    290000, 
     300000, 
-    310000, 
-    320000, 
-    330000, 
-    340000, 
     350000, 
-    360000, 
-    370000, 
-    380000, 
-    390000, 
     400000, 
-    410000, 
-    420000, 
-    430000, 
-    440000, 
     450000, 
-    460000, 
-    470000, 
-    480000, 
-    490000, 
     500000, 
-    510000, 
-    520000, 
-    530000, 
-    540000, 
     550000, 
-    560000, 
-    570000, 
-    580000, 
-    590000, 
     600000, 
-    610000, 
-    620000, 
-    630000, 
-    640000, 
     650000, 
-    660000, 
-    670000, 
-    680000, 
-    690000, 
     700000, 
-    710000, 
-    720000, 
-    730000, 
-    740000, 
     750000, 
-    760000, 
-    770000, 
-    780000, 
-    790000, 
     800000, 
-    810000, 
-    820000, 
-    830000, 
-    840000, 
     850000, 
-    860000, 
-    870000, 
-    880000, 
-    890000, 
     900000, 
-    910000, 
-    920000, 
-    930000, 
-    940000, 
     950000, 
-    960000
+    1000000
 ], 
     "density"  :  [ 
-0, 
-    0.0231, 
-    0.0708, 
-    0.0536, 
-    0.0549, 
-    0.0539, 
-    0.055, 
-    0.0532, 
-    0.0488, 
-    0.0435, 
-    0.0376, 
-    0.0329, 
-    0.0306, 
-    0.0248, 
-    0.0244, 
+0.0232, 
+    0.2882, 
+    0.2159, 
+    0.1227, 
+    0.0776, 
+    0.0538, 
+    0.0405, 
+    0.0308, 
+    0.0235, 
     0.0214, 
-    0.0216, 
-    0.0177, 
-    0.0177, 
-    0.0161, 
-    0.013, 
-    0.013, 
-    0.0121, 
-    0.0105, 
-    0.0113, 
-    0.0103, 
-    0.0095, 
+    0.0173, 
+    0.015, 
+    0.012, 
+    0.011, 
     0.01, 
-    0.0076, 
-    0.008, 
-    0.0075, 
-    0.0075, 
-    0.0068, 
-    0.006, 
-    0.0068, 
-    0.0058, 
-    0.0054, 
-    0.0054, 
-    0.0047, 
-    0.0045, 
-    0.0042, 
-    0.0047, 
-    0.0045, 
-    0.0049, 
-    0.0037, 
-    0.0041, 
-    0.0042, 
-    0.0035, 
-    0.0037, 
-    0.0033, 
-    0.0032, 
-    0.0035, 
-    0.0035, 
-    0.0029, 
-    0.0031, 
-    0.0024, 
-    0.003, 
-    0.0025, 
-    0.0027, 
-    0.0019, 
-    0.0019, 
-    0.003, 
-    0.0024, 
-    0.0017, 
-    0.0028, 
-    0.0021, 
-    0.002, 
-    0.0019, 
-    0.002, 
-    0.0019, 
-    0.0021, 
-    0.002, 
-    0.0016, 
-    0.0017, 
-    0.002, 
-    0.0014, 
-    0.002, 
-    0.0013, 
-    0.0021, 
-    0.0019, 
-    0.0017, 
-    0.0015, 
-    0.0015, 
-    0.001, 
-    0.0011, 
-    0.0018, 
-    0.0009, 
-    0.0009, 
-    0.0016, 
-    0.0016, 
-    0.0013, 
-    0.0009, 
-    0.0011, 
-    0.0012, 
-    0.0012, 
-    0.0016, 
-    0.0011, 
+    0.0087, 
+    0.0085, 
+    0.0063, 
+    0.0064, 
+    0.0062, 
     0.001
 ], 
     "y"  :  [ 
-1, 
-    492, 
-    1506, 
-    1139, 
-    1168, 
-    1146, 
-    1169, 
-    1131, 
-    1037, 
-    925, 
-    799, 
-    700, 
-    650, 
-    528, 
-    518, 
+493, 
+    6128, 
+    4592, 
+    2610, 
+    1650, 
+    1144, 
+    862, 
+    656, 
+    500, 
     455, 
-    459, 
-    377, 
-    377, 
-    342, 
-    277, 
-    277, 
-    258, 
-    224, 
-    241, 
-    220, 
-    201, 
+    368, 
+    318, 
+    255, 
+    234, 
     212, 
-    161, 
-    171, 
-    159, 
-    159, 
-    145, 
-    128, 
-    145, 
-    124, 
-    114, 
-    114, 
-    101, 
-    95, 
-    89, 
-    101, 
-    95, 
-    104, 
-    79, 
-    88, 
-    89, 
-    74, 
-    79, 
-    71, 
-    69, 
-    75, 
-    75, 
-    62, 
-    66, 
-    52, 
-    63, 
-    53, 
-    58, 
-    40, 
-    41, 
-    63, 
-    51, 
-    36, 
-    60, 
-    45, 
-    42, 
-    41, 
-    43, 
-    40, 
-    45, 
-    43, 
-    35, 
-    36, 
-    42, 
-    29, 
-    43, 
-    28, 
-    44, 
-    40, 
-    36, 
-    32, 
-    31, 
-    22, 
-    23, 
-    38, 
-    20, 
-    20, 
-    35, 
-    35, 
-    27, 
-    19, 
-    23, 
-    25, 
-    26, 
-    34, 
-    24, 
+    185, 
+    180, 
+    134, 
+    136, 
+    132, 
     22
 ], 
     "mids"  :  [ 
--15000, 
-    -5000, 
-    5000, 
-    15000, 
+-25000, 
     25000, 
-    35000, 
-    45000, 
-    55000, 
-    65000, 
     75000, 
-    85000, 
-    95000, 
-    105000, 
-    115000, 
     125000, 
-    135000, 
-    145000, 
-    155000, 
-    165000, 
     175000, 
-    185000, 
-    195000, 
-    205000, 
-    215000, 
     225000, 
-    235000, 
-    245000, 
-    255000, 
-    265000, 
     275000, 
-    285000, 
-    295000, 
-    305000, 
-    315000, 
     325000, 
-    335000, 
-    345000, 
-    355000, 
-    365000, 
     375000, 
-    385000, 
-    395000, 
-    405000, 
-    415000, 
     425000, 
-    435000, 
-    445000, 
-    455000, 
-    465000, 
     475000, 
-    485000, 
-    495000, 
-    505000, 
-    515000, 
     525000, 
-    535000, 
-    545000, 
-    555000, 
-    565000, 
     575000, 
-    585000, 
-    595000, 
-    605000, 
-    615000, 
     625000, 
-    635000, 
-    645000, 
-    655000, 
-    665000, 
     675000, 
-    685000, 
-    695000, 
-    705000, 
-    715000, 
     725000, 
-    735000, 
-    745000, 
-    755000, 
-    765000, 
     775000, 
-    785000, 
-    795000, 
-    805000, 
-    815000, 
     825000, 
-    835000, 
-    845000, 
-    855000, 
-    865000, 
     875000, 
-    885000, 
-    895000, 
-    905000, 
-    915000, 
     925000, 
-    935000, 
-    945000, 
-    955000
+    975000
 ], 
     "mean"  :  [ 
 3531376.4064
@@ -5691,8 +4056,10 @@
   {  "STAT" :  "Rows"  ,  "VAL" :  "25,000"  ,  "PER" :  ""  }, 
   {  "STAT" :  "Distinct"  ,  "VAL" :  "19,931"  ,  "PER" :  "(79.7%)"  }, 
   {  "STAT" :  "Missing/NA"  ,  "VAL" :  "1,377"  ,  "PER" :  "(5.5%)"  }, 
-  {  "STAT" :  "Zero"  ,  "VAL" :  "3,257"  ,  "PER" :  "(13%)"  }, 
-  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(13%)"  }
+  {  "STAT" :  "Zero"  ,  "VAL" :  "3,257"  ,  "PER" :  "(13.0%)"  }, 
+  {  "STAT" :  "Most Common"  ,  "VAL" :  "0"  ,  "PER" :  "(13.0%)"  }, 
+  {  "STAT" :  "Skew"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }, 
+  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "HIGH"  ,  "PER" :  ""  }
 ]</t>
   </si>
   <si>
@@ -5716,122 +4083,30 @@
     <t xml:space="preserve">  { 
     "breaks"  :  [ 
 -300000, 
-    -290000, 
-    -280000, 
-    -270000, 
-    -260000, 
     -250000, 
-    -240000, 
-    -230000, 
-    -220000, 
-    -210000, 
     -200000, 
-    -190000, 
-    -180000, 
-    -170000, 
-    -160000, 
     -150000, 
-    -140000, 
-    -130000, 
-    -120000, 
-    -110000, 
     -100000, 
-    -90000, 
-    -80000, 
-    -70000, 
-    -60000, 
     -50000, 
-    -40000, 
-    -30000, 
-    -20000, 
-    -10000, 
     0, 
-    10000, 
-    20000, 
-    30000, 
-    40000, 
     50000, 
-    60000, 
-    70000, 
-    80000, 
-    90000, 
     100000, 
-    110000, 
-    120000, 
-    130000, 
-    140000, 
     150000, 
-    160000, 
-    170000, 
-    180000, 
-    190000, 
     200000, 
-    210000, 
-    220000, 
-    230000, 
-    240000, 
     250000, 
-    260000, 
-    270000, 
-    280000, 
-    290000, 
     300000, 
-    310000, 
-    320000, 
-    330000, 
-    340000, 
     350000, 
-    360000, 
-    370000, 
-    380000, 
-    390000, 
     400000, 
-    410000, 
-    420000, 
-    430000, 
-    440000, 
     450000, 
-    460000, 
-    470000, 
-    480000, 
-    490000, 
     500000, 
-    510000, 
-    520000, 
-    530000, 
-    540000, 
     550000, 
-    560000, 
-    570000, 
-    580000, 
-    590000, 
     600000, 
-    610000, 
-    620000, 
-    630000, 
-    640000, 
     650000, 
-    660000, 
-    670000, 
-    680000, 
-    690000, 
     700000, 
-    710000, 
-    720000, 
-    730000, 
-    740000, 
     750000, 
-    760000, 
-    770000, 
-    780000, 
-    790000, 
     800000, 
-    810000, 
-    820000, 
-    830000, 
-    840000, 
     850000, 
-    860000
+    900000
 ], 
     "density"  :  [ 
 0, 
@@ -5839,353 +4114,77 @@
     0, 
     0, 
     0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
     0.1623, 
-    0.0478, 
-    0.0396, 
-    0.0444, 
-    0.0465, 
-    0.0469, 
-    0.0464, 
-    0.0442, 
-    0.0373, 
-    0.0335, 
-    0.0312, 
-    0.025, 
-    0.0245, 
-    0.0229, 
-    0.0193, 
-    0.0174, 
-    0.0162, 
-    0.0154, 
-    0.0165, 
-    0.0121, 
-    0.0122, 
-    0.0112, 
-    0.01, 
-    0.0105, 
-    0.0099, 
-    0.0083, 
-    0.0076, 
-    0.0073, 
-    0.0084, 
-    0.007, 
-    0.0064, 
-    0.0066, 
-    0.0055, 
-    0.0059, 
-    0.0054, 
-    0.0053, 
-    0.0041, 
-    0.0042, 
-    0.0048, 
-    0.0032, 
-    0.0042, 
-    0.004, 
-    0.0038, 
-    0.0035, 
-    0.0043, 
-    0.0039, 
-    0.0042, 
-    0.0031, 
-    0.0031, 
-    0.0027, 
-    0.0026, 
-    0.0034, 
-    0.0022, 
-    0.003, 
-    0.0023, 
-    0.0024, 
-    0.002, 
-    0.0023, 
-    0.002, 
-    0.0019, 
-    0.0019, 
-    0.0024, 
-    0.0018, 
-    0.0023, 
-    0.002, 
-    0.0022, 
-    0.0014, 
-    0.0018, 
-    0.0017, 
-    0.0021, 
-    0.0017, 
-    0.0017, 
-    0.0014, 
-    0.0016, 
-    0.0014, 
-    0.0018, 
-    0.0019, 
-    0.0011, 
-    0.0014, 
-    0.0013, 
-    0.0017, 
-    0.0018, 
-    0.0014, 
-    0.0014, 
-    0.0012, 
-    0.0013, 
+    0.2252, 
+    0.1926, 
+    0.1091, 
+    0.0725, 
+    0.0498, 
+    0.0366, 
+    0.0287, 
+    0.0205, 
+    0.0195, 
+    0.0157, 
+    0.0134, 
+    0.0102, 
+    0.0108, 
+    0.0088, 
+    0.008, 
+    0.0074, 
+    0.0072, 
     0.0015
 ], 
     "y"  :  [ 
 1, 
     0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
+    1, 
     0, 
     1, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    0, 
-    1, 
-    0, 
-    0, 
-    0, 
-    0, 
     3259, 
-    961, 
-    796, 
-    891, 
-    933, 
-    942, 
-    932, 
-    887, 
-    750, 
-    673, 
-    627, 
-    503, 
-    493, 
-    460, 
-    387, 
-    349, 
-    326, 
-    309, 
-    332, 
-    244, 
-    246, 
-    224, 
-    201, 
-    210, 
-    198, 
-    167, 
-    153, 
-    146, 
-    169, 
-    140, 
-    128, 
-    132, 
-    111, 
-    118, 
-    108, 
-    107, 
-    83, 
-    85, 
-    96, 
-    64, 
-    84, 
-    80, 
-    77, 
-    70, 
-    86, 
-    79, 
-    84, 
-    63, 
-    62, 
-    54, 
-    53, 
-    69, 
-    44, 
-    60, 
-    47, 
-    49, 
-    41, 
-    47, 
-    40, 
-    39, 
-    38, 
-    48, 
-    36, 
-    47, 
-    40, 
-    45, 
-    28, 
-    37, 
-    34, 
-    42, 
-    35, 
-    34, 
-    29, 
-    32, 
-    28, 
-    37, 
-    38, 
-    22, 
-    28, 
-    26, 
-    34, 
-    37, 
-    28, 
-    28, 
-    25, 
-    27, 
+    4523, 
+    3869, 
+    2192, 
+    1457, 
+    1000, 
+    736, 
+    576, 
+    412, 
+    392, 
+    316, 
+    269, 
+    205, 
+    216, 
+    176, 
+    160, 
+    148, 
+    145, 
     31
 ], 
     "mids"  :  [ 
--295000, 
-    -285000, 
-    -275000, 
-    -265000, 
-    -255000, 
-    -245000, 
-    -235000, 
+-275000, 
     -225000, 
-    -215000, 
-    -205000, 
-    -195000, 
-    -185000, 
     -175000, 
-    -165000, 
-    -155000, 
-    -145000, 
-    -135000, 
     -125000, 
-    -115000, 
-    -105000, 
-    -95000, 
-    -85000, 
     -75000, 
-    -65000, 
-    -55000, 
-    -45000, 
-    -35000, 
     -25000, 
-    -15000, 
-    -5000, 
-    5000, 
-    15000, 
     25000, 
-    35000, 
-    45000, 
-    55000, 
-    65000, 
     75000, 
-    85000, 
-    95000, 
-    105000, 
-    115000, 
     125000, 
-    135000, 
-    145000, 
-    155000, 
-    165000, 
     175000, 
-    185000, 
-    195000, 
-    205000, 
-    215000, 
     225000, 
-    235000, 
-    245000, 
-    255000, 
-    265000, 
     275000, 
-    285000, 
-    295000, 
-    305000, 
-    315000, 
     325000, 
-    335000, 
-    345000, 
-    355000, 
-    365000, 
     375000, 
-    385000, 
-    395000, 
-    405000, 
-    415000, 
     425000, 
-    435000, 
-    445000, 
-    455000, 
-    465000, 
     475000, 
-    485000, 
-    495000, 
-    505000, 
-    515000, 
     525000, 
-    535000, 
-    545000, 
-    555000, 
-    565000, 
     575000, 
-    585000, 
-    595000, 
-    605000, 
-    615000, 
     625000, 
-    635000, 
-    645000, 
-    655000, 
-    665000, 
     675000, 
-    685000, 
-    695000, 
-    705000, 
-    715000, 
     725000, 
-    735000, 
-    745000, 
-    755000, 
-    765000, 
     775000, 
-    785000, 
-    795000, 
-    805000, 
-    815000, 
     825000, 
-    835000, 
-    845000, 
-    855000
+    875000
 ], 
     "mean"  :  [ 
 3407085.2205

</xml_diff>

<commit_message>
Regenerate working-example DGFs + guides under read-as-text
Rebuilds DGF, DGF-V2, and DGF-temporal-demo (and re-renders all three guides)
with create_dgf(read_as_text = TRUE): every raw_data_storage is now "character"
and safe-numeric columns are promoted. The curated DGF-V2 now retypes the census
tract to identifier/geographic_id via the full create_dgf + retype_dgf recipe
(the earlier committed copy used the base-R fallback that left it a number).
Confirmed create_dgf runs on the 25k demo via the installed package - the
earlier segfaults were load_all-specific, not create_dgf itself.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working-example/DGF-V2.xlsx
+++ b/working-example/DGF-V2.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DGF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -101,13 +101,13 @@
     <t xml:space="preserve">F9_00_ORG_NAME_L1</t>
   </si>
   <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
     <t xml:space="preserve">Organization name</t>
   </si>
   <si>
     <t xml:space="preserve">Legal name of the filing organization (Form 990, header).</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">character</t>
@@ -713,7 +713,7 @@
     <t xml:space="preserve">IRS-assigned 9-digit taxpayer ID; the unique key for the organization.</t>
   </si>
   <si>
-    <t xml:space="preserve">numeric</t>
+    <t xml:space="preserve">TRUE</t>
   </si>
   <si>
     <t xml:space="preserve">113161527 ;; 
@@ -721,6 +721,9 @@
 751627109 ;; 
 61636713 ;; 
 542015951</t>
+  </si>
+  <si>
+    <t xml:space="preserve">numeric</t>
   </si>
   <si>
     <t xml:space="preserve">identifier</t>
@@ -1873,243 +1876,45 @@
     <t xml:space="preserve">11001010700 ;; 48201531700 ;; 6037294421 ;; 11001010100 ;; 11001005800 ;; 17031839100 ;; 6067001101 ;; 6073020809 ;; 48113020300 ;; 11001005900 ;; 18097391000 ;; 4013941000 ;; 51510201900 ;; 6085512100 ;; 36061016100 ;; 42003020100 ;; 48453000102 ;; 48453001100 ;; 6075011700 ;; 11001006202 ;; 39049004000 ;; 17031320100 ;; 42003191100 ;; 1097003707 ;; 6075061500 ;; 22033003501 ;; 28049010500 ;; 350</t>
   </si>
   <si>
-    <t xml:space="preserve">[ 
-  {  "STAT" :  "Minimum"  ,  "VAL" :  "1,001,020,500"  }, 
-  {  "STAT" :  "Q - 05"  ,  "VAL" :  "6,029,003,250"  }, 
-  {  "STAT" :  "Q - 25"  ,  "VAL" :  "17,031,320,100"  }, 
-  {  "STAT" :  "Median"  ,  "VAL" :  "28,012,950,350"  }, 
-  {  "STAT" :  "Mean"  ,  "VAL" :  "28,488,147,053"  }, 
-  {  "STAT" :  "Q - 75"  ,  "VAL" :  "41,051,008,202"  }, 
-  {  "STAT" :  "Q - 95"  ,  "VAL" :  "53,033,008,055"  }, 
-  {  "STAT" :  "Maximum"  ,  "VAL" :  "5.6043e+10"  }, 
-  {  "STAT" :  "Skew"  ,  "VAL" :  "-0.02"  }, 
-  {  "STAT" :  "Kurtosis"  ,  "VAL" :  "-1.17"  }
-]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  { 
-    "breaks"  :  [ 
-6029003306, 
-    6969083399.9, 
-    7909163493.8, 
-    8849243587.7, 
-    9789323681.6, 
-    10729403775.5, 
-    11669483869.4, 
-    12609563963.3, 
-    13549644057.2, 
-    14489724151.1, 
-    15429804245, 
-    16369884338.9, 
-    17309964432.8, 
-    18250044526.7, 
-    19190124620.6, 
-    20130204714.5, 
-    21070284808.4, 
-    22010364902.3, 
-    22950444996.2, 
-    23890525090.1, 
-    24830605184, 
-    25770685277.9, 
-    26710765371.8, 
-    27650845465.7, 
-    28590925559.6, 
-    29531005653.5, 
-    30471085747.4, 
-    31411165841.3, 
-    32351245935.2, 
-    33291326029.1, 
-    34231406123, 
-    35171486216.9, 
-    36111566310.8, 
-    37051646404.7, 
-    37991726498.6, 
-    38931806592.5, 
-    39871886686.4, 
-    40811966780.3, 
-    41752046874.2, 
-    42692126968.1, 
-    43632207062, 
-    44572287155.9, 
-    45512367249.8, 
-    46452447343.7, 
-    47392527437.6, 
-    48332607531.5, 
-    49272687625.4, 
-    50212767719.3, 
-    51152847813.2, 
-    52092927907.1, 
-    53033008001
-], 
-    "density"  :  [ 
-0.0869, 
-    0, 
-    0.0192, 
-    0.0177, 
-    0.0044, 
-    0.0142, 
-    0.0401, 
-    0.0232, 
-    0, 
-    0.0041, 
-    0.0054, 
-    0.0531, 
-    0.0345, 
-    0.0193, 
-    0.008, 
-    0.0112, 
-    0.0109, 
-    0.0134, 
-    0.0074, 
-    0.0221, 
-    0.0341, 
-    0.0391, 
-    0.031, 
-    0.0111, 
-    0.0257, 
-    0.0071, 
-    0.0093, 
-    0.0053, 
-    0.0066, 
-    0.0342, 
-    0.0059, 
-    0.0642, 
-    0.0127, 
-    0.019, 
-    0.0059, 
-    0.049, 
-    0.0117, 
-    0.0146, 
-    0.0606, 
-    0, 
-    0.0061, 
-    0.0118, 
-    0.0058, 
-    0.0175, 
-    0.0459, 
-    0.0271, 
-    0.0047, 
-    0.0151, 
-    0.0156, 
-    0.008
-], 
-    "y"  :  [ 
-1711, 
-    0, 
-    379, 
-    348, 
-    87, 
-    280, 
-    789, 
-    458, 
-    0, 
-    81, 
-    107, 
-    1046, 
-    679, 
-    381, 
-    157, 
-    221, 
-    215, 
-    263, 
-    146, 
-    435, 
-    672, 
-    771, 
-    611, 
-    218, 
-    506, 
-    139, 
-    184, 
-    104, 
-    130, 
-    673, 
-    116, 
-    1265, 
-    250, 
-    375, 
-    117, 
-    965, 
-    231, 
-    288, 
-    1194, 
-    0, 
-    121, 
-    233, 
-    114, 
-    345, 
-    905, 
-    534, 
-    92, 
-    298, 
-    308, 
-    158
-], 
-    "mids"  :  [ 
-6499043352.95, 
-    7439123446.85, 
-    8379203540.75, 
-    9319283634.65, 
-    10259363728.55, 
-    11199443822.45, 
-    12139523916.35, 
-    13079604010.25, 
-    14019684104.15, 
-    14959764198.05, 
-    15899844291.95, 
-    16839924385.85, 
-    17780004479.75, 
-    18720084573.65, 
-    19660164667.55, 
-    20600244761.45, 
-    21540324855.35, 
-    22480404949.25, 
-    23420485043.15, 
-    24360565137.05, 
-    25300645230.95, 
-    26240725324.85, 
-    27180805418.75, 
-    28120885512.65, 
-    29060965606.55, 
-    30001045700.45, 
-    30941125794.35, 
-    31881205888.25, 
-    32821285982.15, 
-    33761366076.05, 
-    34701446169.95, 
-    35641526263.85, 
-    36581606357.75, 
-    37521686451.65, 
-    38461766545.55, 
-    39401846639.45, 
-    40341926733.35, 
-    41282006827.25, 
-    42222086921.15, 
-    43162167015.05, 
-    44102247108.95, 
-    45042327202.85, 
-    45982407296.75, 
-    46922487390.65, 
-    47862567484.55, 
-    48802647578.45, 
-    49742727672.35, 
-    50682807766.25, 
-    51622887860.15, 
-    52562967954.05
-], 
-    "mean"  :  [ 
-28488147052.6496
-], 
-    "median"  :  [ 
-28012950350
-], 
-    "min"  :  [ 
-1001020500
-], 
-    "max"  :  [ 
-56043000200
-]
-  }</t>
+    <t xml:space="preserve">{
+  "STATS": [
+    {
+      "STAT": "Distinct",
+      "VAL": 14264
+    },
+    {
+      "STAT": "Duplicated",
+      "VAL": 7626
+    }
+  ],
+  "HIST": [],
+  "COMMON": [
+    {
+      "Value": "11001010700",
+      "Frequency": 69
+    },
+    {
+      "Value": "48201531700",
+      "Frequency": 63
+    },
+    {
+      "Value": "6037294421",
+      "Frequency": 36
+    },
+    {
+      "Value": "11001010100",
+      "Frequency": 34
+    },
+    {
+      "Value": "11001005800",
+      "Frequency": 32
+    },
+    {
+      "Value": "17031839100",
+      "Frequency": 31
+    }
+  ]
+}</t>
   </si>
   <si>
     <t xml:space="preserve">afbc196795d8aeaf02161da0a2f65571</t>
@@ -2182,6 +1987,12 @@
 201905</t>
   </si>
   <si>
+    <t xml:space="preserve">month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">temporal</t>
+  </si>
+  <si>
     <t xml:space="preserve">reporting_period</t>
   </si>
   <si>
@@ -2195,65 +2006,53 @@
   </si>
   <si>
     <t xml:space="preserve">[ 
-  {  "Value" :  "201912"  ,  "Frequency" :  9884  }, 
-  {  "Value" :  "201812"  ,  "Frequency" :  3477  }, 
-  {  "Value" :  "201906"  ,  "Frequency" :  2064  }, 
-  {  "Value" :  "201712"  ,  "Frequency" :  1626  }, 
-  {  "Value" :  "202006"  ,  "Frequency" :  1312  }, 
-  {  "Value" :  "201806"  ,  "Frequency" :  840  }, 
-  {  "Value" :  "201909"  ,  "Frequency" :  812  }, 
-  {  "Value" :  "201908"  ,  "Frequency" :  406  }, 
-  {  "Value" :  "201706"  ,  "Frequency" :  362  }, 
-  {  "Value" :  "201903"  ,  "Frequency" :  356  }, 
-  {  "Value" :  "202003"  ,  "Frequency" :  352  }, 
-  {  "Value" :  "201905"  ,  "Frequency" :  326  }, 
-  {  "Value" :  "201904"  ,  "Frequency" :  278  }, 
-  {  "Value" :  "201910"  ,  "Frequency" :  272  }, 
-  {  "Value" :  "202005"  ,  "Frequency" :  252  }, 
-  {  "Value" :  "201809"  ,  "Frequency" :  244  }, 
-  {  "Value" :  "202004"  ,  "Frequency" :  183  }, 
-  {  "Value" :  "201907"  ,  "Frequency" :  161  }, 
-  {  "Value" :  "201805"  ,  "Frequency" :  154  }, 
-  {  "Value" :  "201808"  ,  "Frequency" :  139  }, 
-  {  "Value" :  "201911"  ,  "Frequency" :  123  }, 
-  {  "Value" :  "201709"  ,  "Frequency" :  121  }, 
-  {  "Value" :  "201803"  ,  "Frequency" :  110  }, 
-  {  "Value" :  "201804"  ,  "Frequency" :  102  }, 
-  {  "Value" :  "201810"  ,  "Frequency" :  94  }, 
-  {  "Value" :  "202007"  ,  "Frequency" :  91  }, 
-  {  "Value" :  "202008"  ,  "Frequency" :  79  }, 
-  {  "Value" :  "202009"  ,  "Frequency" :  74  }, 
-  {  "Value" :  "202001"  ,  "Frequency" :  66  }, 
-  {  "Value" :  "201807"  ,  "Frequency" :  65  }, 
-  {  "Value" :  "201705"  ,  "Frequency" :  64  }, 
-  {  "Value" :  "201708"  ,  "Frequency" :  64  }, 
-  {  "Value" :  "202002"  ,  "Frequency" :  59  }, 
-  {  "Value" :  "201902"  ,  "Frequency" :  57  }, 
-  {  "Value" :  "201704"  ,  "Frequency" :  46  }, 
-  {  "Value" :  "201710"  ,  "Frequency" :  46  }, 
-  {  "Value" :  "201811"  ,  "Frequency" :  46  }, 
-  {  "Value" :  "201901"  ,  "Frequency" :  34  }, 
-  {  "Value" :  "201707"  ,  "Frequency" :  32  }, 
-  {  "Value" :  "201802"  ,  "Frequency" :  32  }, 
-  {  "Value" :  "201703"  ,  "Frequency" :  31  }, 
-  {  "Value" :  "201711"  ,  "Frequency" :  25  }, 
-  {  "Value" :  "202010"  ,  "Frequency" :  13  }, 
-  {  "Value" :  "201801"  ,  "Frequency" :  9  }, 
-  {  "Value" :  "201701"  ,  "Frequency" :  8  }, 
-  {  "Value" :  "201702"  ,  "Frequency" :  8  }, 
-  {  "Value" :  "202011"  ,  "Frequency" :  1  }
-]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 
-  {  "x" :  "201912"  ,  "Freq" :  9884  }, 
-  {  "x" :  "201812"  ,  "Freq" :  3477  }, 
-  {  "x" :  "201906"  ,  "Freq" :  2064  }, 
-  {  "x" :  "201712"  ,  "Freq" :  1626  }, 
-  {  "x" :  "202006"  ,  "Freq" :  1312  }, 
-  {  "x" :  "201806"  ,  "Freq" :  840  }, 
-  {  "x" :  "201909"  ,  "Freq" :  812  }, 
-  {  "x" :  "other"  ,  "Freq" :  4985  }
+  {  "Value" :  "201701"  ,  "Count" :  8  }, 
+  {  "Value" :  "201702"  ,  "Count" :  8  }, 
+  {  "Value" :  "201703"  ,  "Count" :  31  }, 
+  {  "Value" :  "201704"  ,  "Count" :  46  }, 
+  {  "Value" :  "201705"  ,  "Count" :  64  }, 
+  {  "Value" :  "201706"  ,  "Count" :  362  }, 
+  {  "Value" :  "201707"  ,  "Count" :  32  }, 
+  {  "Value" :  "201708"  ,  "Count" :  64  }, 
+  {  "Value" :  "201709"  ,  "Count" :  121  }, 
+  {  "Value" :  "201710"  ,  "Count" :  46  }, 
+  {  "Value" :  "201711"  ,  "Count" :  25  }, 
+  {  "Value" :  "201712"  ,  "Count" :  1626  }, 
+  {  "Value" :  "201801"  ,  "Count" :  9  }, 
+  {  "Value" :  "201802"  ,  "Count" :  32  }, 
+  {  "Value" :  "201803"  ,  "Count" :  110  }, 
+  {  "Value" :  "201804"  ,  "Count" :  102  }, 
+  {  "Value" :  "201805"  ,  "Count" :  154  }, 
+  {  "Value" :  "201806"  ,  "Count" :  840  }, 
+  {  "Value" :  "201807"  ,  "Count" :  65  }, 
+  {  "Value" :  "201808"  ,  "Count" :  139  }, 
+  {  "Value" :  "201809"  ,  "Count" :  244  }, 
+  {  "Value" :  "201810"  ,  "Count" :  94  }, 
+  {  "Value" :  "201811"  ,  "Count" :  46  }, 
+  {  "Value" :  "201812"  ,  "Count" :  3477  }, 
+  {  "Value" :  "201901"  ,  "Count" :  34  }, 
+  {  "Value" :  "201902"  ,  "Count" :  57  }, 
+  {  "Value" :  "201903"  ,  "Count" :  356  }, 
+  {  "Value" :  "201904"  ,  "Count" :  278  }, 
+  {  "Value" :  "201905"  ,  "Count" :  326  }, 
+  {  "Value" :  "201906"  ,  "Count" :  2064  }, 
+  {  "Value" :  "201907"  ,  "Count" :  161  }, 
+  {  "Value" :  "201908"  ,  "Count" :  406  }, 
+  {  "Value" :  "201909"  ,  "Count" :  812  }, 
+  {  "Value" :  "201910"  ,  "Count" :  272  }, 
+  {  "Value" :  "201911"  ,  "Count" :  123  }, 
+  {  "Value" :  "201912"  ,  "Count" :  9884  }, 
+  {  "Value" :  "202001"  ,  "Count" :  66  }, 
+  {  "Value" :  "202002"  ,  "Count" :  59  }, 
+  {  "Value" :  "202003"  ,  "Count" :  352  }, 
+  {  "Value" :  "202004"  ,  "Count" :  183  }, 
+  {  "Value" :  "202005"  ,  "Count" :  252  }, 
+  {  "Value" :  "202006"  ,  "Count" :  1312  }, 
+  {  "Value" :  "202007"  ,  "Count" :  91  }, 
+  {  "Value" :  "202008"  ,  "Count" :  79  }, 
+  {  "Value" :  "202009"  ,  "Count" :  74  }, 
+  {  "Value" :  "202010"  ,  "Count" :  13  }, 
+  {  "Value" :  "202011"  ,  "Count" :  1  }
 ]</t>
   </si>
   <si>
@@ -2337,64 +2136,52 @@
   </si>
   <si>
     <t xml:space="preserve">[ 
-  {  "Value" :  "201812"  ,  "Frequency" :  9298  }, 
-  {  "Value" :  "201712"  ,  "Frequency" :  3002  }, 
-  {  "Value" :  "201806"  ,  "Frequency" :  1767  }, 
-  {  "Value" :  "201906"  ,  "Frequency" :  1060  }, 
-  {  "Value" :  "201809"  ,  "Frequency" :  744  }, 
-  {  "Value" :  "201706"  ,  "Frequency" :  539  }, 
-  {  "Value" :  "201612"  ,  "Frequency" :  478  }, 
-  {  "Value" :  "201808"  ,  "Frequency" :  370  }, 
-  {  "Value" :  "201803"  ,  "Frequency" :  321  }, 
-  {  "Value" :  "201903"  ,  "Frequency" :  319  }, 
-  {  "Value" :  "201805"  ,  "Frequency" :  265  }, 
-  {  "Value" :  "201810"  ,  "Frequency" :  255  }, 
-  {  "Value" :  "201804"  ,  "Frequency" :  246  }, 
-  {  "Value" :  "201905"  ,  "Frequency" :  206  }, 
-  {  "Value" :  "201709"  ,  "Frequency" :  195  }, 
-  {  "Value" :  "201606"  ,  "Frequency" :  164  }, 
-  {  "Value" :  "201904"  ,  "Frequency" :  162  }, 
-  {  "Value" :  "201807"  ,  "Frequency" :  123  }, 
-  {  "Value" :  "201811"  ,  "Frequency" :  122  }, 
-  {  "Value" :  "201708"  ,  "Frequency" :  101  }, 
-  {  "Value" :  "201705"  ,  "Frequency" :  90  }, 
-  {  "Value" :  "201710"  ,  "Frequency" :  88  }, 
-  {  "Value" :  "201704"  ,  "Frequency" :  64  }, 
-  {  "Value" :  "201901"  ,  "Frequency" :  61  }, 
-  {  "Value" :  "201907"  ,  "Frequency" :  58  }, 
-  {  "Value" :  "201703"  ,  "Frequency" :  51  }, 
-  {  "Value" :  "201902"  ,  "Frequency" :  49  }, 
-  {  "Value" :  "201802"  ,  "Frequency" :  46  }, 
-  {  "Value" :  "201908"  ,  "Frequency" :  44  }, 
-  {  "Value" :  "201909"  ,  "Frequency" :  42  }, 
-  {  "Value" :  "201711"  ,  "Frequency" :  41  }, 
-  {  "Value" :  "201707"  ,  "Frequency" :  39  }, 
-  {  "Value" :  "201605"  ,  "Frequency" :  36  }, 
-  {  "Value" :  "201609"  ,  "Frequency" :  34  }, 
-  {  "Value" :  "201801"  ,  "Frequency" :  29  }, 
-  {  "Value" :  "201604"  ,  "Frequency" :  27  }, 
-  {  "Value" :  "201608"  ,  "Frequency" :  23  }, 
-  {  "Value" :  "201702"  ,  "Frequency" :  22  }, 
-  {  "Value" :  "201603"  ,  "Frequency" :  18  }, 
-  {  "Value" :  "201607"  ,  "Frequency" :  16  }, 
-  {  "Value" :  "201610"  ,  "Frequency" :  13  }, 
-  {  "Value" :  "201611"  ,  "Frequency" :  9  }, 
-  {  "Value" :  "201910"  ,  "Frequency" :  7  }, 
-  {  "Value" :  "201601"  ,  "Frequency" :  5  }, 
-  {  "Value" :  "201602"  ,  "Frequency" :  4  }, 
-  {  "Value" :  "201701"  ,  "Frequency" :  3  }
-]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[ 
-  {  "x" :  "201812"  ,  "Freq" :  9298  }, 
-  {  "x" :  "201712"  ,  "Freq" :  3002  }, 
-  {  "x" :  "201806"  ,  "Freq" :  1767  }, 
-  {  "x" :  "201906"  ,  "Freq" :  1060  }, 
-  {  "x" :  "201809"  ,  "Freq" :  744  }, 
-  {  "x" :  "201706"  ,  "Freq" :  539  }, 
-  {  "x" :  "201612"  ,  "Freq" :  478  }, 
-  {  "x" :  "other"  ,  "Freq" :  3768  }
+  {  "Value" :  "201601"  ,  "Count" :  5  }, 
+  {  "Value" :  "201602"  ,  "Count" :  4  }, 
+  {  "Value" :  "201603"  ,  "Count" :  18  }, 
+  {  "Value" :  "201604"  ,  "Count" :  27  }, 
+  {  "Value" :  "201605"  ,  "Count" :  36  }, 
+  {  "Value" :  "201606"  ,  "Count" :  164  }, 
+  {  "Value" :  "201607"  ,  "Count" :  16  }, 
+  {  "Value" :  "201608"  ,  "Count" :  23  }, 
+  {  "Value" :  "201609"  ,  "Count" :  34  }, 
+  {  "Value" :  "201610"  ,  "Count" :  13  }, 
+  {  "Value" :  "201611"  ,  "Count" :  9  }, 
+  {  "Value" :  "201612"  ,  "Count" :  478  }, 
+  {  "Value" :  "201701"  ,  "Count" :  3  }, 
+  {  "Value" :  "201702"  ,  "Count" :  22  }, 
+  {  "Value" :  "201703"  ,  "Count" :  51  }, 
+  {  "Value" :  "201704"  ,  "Count" :  64  }, 
+  {  "Value" :  "201705"  ,  "Count" :  90  }, 
+  {  "Value" :  "201706"  ,  "Count" :  539  }, 
+  {  "Value" :  "201707"  ,  "Count" :  39  }, 
+  {  "Value" :  "201708"  ,  "Count" :  101  }, 
+  {  "Value" :  "201709"  ,  "Count" :  195  }, 
+  {  "Value" :  "201710"  ,  "Count" :  88  }, 
+  {  "Value" :  "201711"  ,  "Count" :  41  }, 
+  {  "Value" :  "201712"  ,  "Count" :  3002  }, 
+  {  "Value" :  "201801"  ,  "Count" :  29  }, 
+  {  "Value" :  "201802"  ,  "Count" :  46  }, 
+  {  "Value" :  "201803"  ,  "Count" :  321  }, 
+  {  "Value" :  "201804"  ,  "Count" :  246  }, 
+  {  "Value" :  "201805"  ,  "Count" :  265  }, 
+  {  "Value" :  "201806"  ,  "Count" :  1767  }, 
+  {  "Value" :  "201807"  ,  "Count" :  123  }, 
+  {  "Value" :  "201808"  ,  "Count" :  370  }, 
+  {  "Value" :  "201809"  ,  "Count" :  744  }, 
+  {  "Value" :  "201810"  ,  "Count" :  255  }, 
+  {  "Value" :  "201811"  ,  "Count" :  122  }, 
+  {  "Value" :  "201812"  ,  "Count" :  9298  }, 
+  {  "Value" :  "201901"  ,  "Count" :  61  }, 
+  {  "Value" :  "201902"  ,  "Count" :  49  }, 
+  {  "Value" :  "201903"  ,  "Count" :  319  }, 
+  {  "Value" :  "201904"  ,  "Count" :  162  }, 
+  {  "Value" :  "201905"  ,  "Count" :  206  }, 
+  {  "Value" :  "201906"  ,  "Count" :  1060  }, 
+  {  "Value" :  "201907"  ,  "Count" :  58  }, 
+  {  "Value" :  "201908"  ,  "Count" :  44  }, 
+  {  "Value" :  "201909"  ,  "Count" :  42  }, 
+  {  "Value" :  "201910"  ,  "Count" :  7  }
 ]</t>
   </si>
   <si>
@@ -4161,21 +3948,65 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Calibri Light"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI Black"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI Black"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Console"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri Light"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF44546A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF833C0C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE3E7ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF2EC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -4190,8 +4021,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4481,1872 +4345,2442 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="20.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="20.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="20.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="20.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="20.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="20.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="20.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="20.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="20.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="20.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="20.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="20.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="20.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="20.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="20.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="20.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="20.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="20.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="20.71" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="20.71" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="20.71" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="20.71" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="20.71" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="20.71" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="20.71" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="20.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B2"/>
-      <c r="C2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F2"/>
-      <c r="G2" t="s">
+      <c r="E2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H2"/>
-      <c r="I2" t="s">
+      <c r="H2" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J2" t="b">
+      <c r="J2" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K2"/>
-      <c r="L2" t="s">
+      <c r="K2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2" t="s">
+      <c r="M2" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="V2" t="s">
+      <c r="V2" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="X2" t="n">
+      <c r="X2" s="7" t="n">
         <v>97</v>
       </c>
-      <c r="Y2"/>
-      <c r="Z2"/>
-      <c r="AA2"/>
-      <c r="AB2" t="s">
+      <c r="Y2" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z2" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA2" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB2" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s">
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B3"/>
-      <c r="C3" t="s">
+      <c r="B3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3"/>
-      <c r="G3" t="s">
+      <c r="E3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H3"/>
-      <c r="I3" t="s">
+      <c r="H3" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="J3" t="b">
+      <c r="J3" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K3"/>
-      <c r="L3" t="s">
+      <c r="K3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="M3"/>
-      <c r="N3"/>
-      <c r="O3"/>
-      <c r="P3" t="s">
+      <c r="M3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="T3" t="s">
+      <c r="T3" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="U3" t="s">
+      <c r="U3" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="V3" t="s">
+      <c r="V3" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="X3" t="n">
+      <c r="X3" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="Y3"/>
-      <c r="Z3"/>
-      <c r="AA3"/>
-      <c r="AB3" t="s">
+      <c r="Y3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB3" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s">
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B4"/>
-      <c r="C4" t="s">
+      <c r="B4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4"/>
-      <c r="G4" t="s">
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H4"/>
-      <c r="I4" t="s">
+      <c r="H4" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="J4" t="b">
+      <c r="J4" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K4"/>
-      <c r="L4" t="s">
+      <c r="K4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="M4"/>
-      <c r="N4"/>
-      <c r="O4"/>
-      <c r="P4" t="s">
+      <c r="M4" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="R4" t="s">
+      <c r="R4" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="S4" t="s">
+      <c r="S4" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="T4" t="s">
+      <c r="T4" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="U4" t="s">
+      <c r="U4" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="V4" t="s">
+      <c r="V4" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="W4" t="s">
+      <c r="W4" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="X4" t="n">
+      <c r="X4" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="Y4"/>
-      <c r="Z4"/>
-      <c r="AA4"/>
-      <c r="AB4" t="s">
+      <c r="Y4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB4" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s">
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B5"/>
-      <c r="C5" t="s">
+      <c r="B5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5"/>
-      <c r="G5" t="s">
+      <c r="E5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H5"/>
-      <c r="I5" t="s">
+      <c r="H5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="J5" t="b">
+      <c r="J5" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K5"/>
-      <c r="L5" t="s">
+      <c r="K5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L5" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="M5"/>
-      <c r="N5"/>
-      <c r="O5"/>
-      <c r="P5" t="s">
+      <c r="M5" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P5" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="Q5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="R5" t="s">
+      <c r="R5" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="S5" t="s">
+      <c r="S5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="T5" t="s">
+      <c r="T5" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="U5" t="s">
+      <c r="U5" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="V5" t="s">
+      <c r="V5" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="W5" t="s">
+      <c r="W5" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="X5" t="n">
+      <c r="X5" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="Y5"/>
-      <c r="Z5"/>
-      <c r="AA5"/>
-      <c r="AB5" t="s">
+      <c r="Y5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB5" s="7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="s">
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B6"/>
-      <c r="C6" t="s">
+      <c r="B6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6"/>
-      <c r="G6" t="s">
+      <c r="E6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="H6"/>
-      <c r="I6" t="s">
+      <c r="G6" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="J6" t="b">
+      <c r="J6" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K6"/>
-      <c r="L6" t="s">
-        <v>77</v>
-      </c>
-      <c r="M6"/>
-      <c r="N6"/>
-      <c r="O6"/>
-      <c r="P6" t="s">
+      <c r="K6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L6" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="M6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P6" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="R6" t="s">
+      <c r="Q6" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="S6" t="s">
+      <c r="R6" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="S6" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="T6" t="s">
-        <v>82</v>
-      </c>
-      <c r="U6" t="s">
+      <c r="T6" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="V6" t="s">
+      <c r="U6" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="W6" t="s">
-        <v>31</v>
-      </c>
-      <c r="X6" t="n">
+      <c r="V6" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="W6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="Y6"/>
-      <c r="Z6"/>
-      <c r="AA6"/>
-      <c r="AB6" t="s">
-        <v>85</v>
+      <c r="Y6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB6" s="7" t="s">
+        <v>86</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7"/>
-      <c r="C7" t="s">
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D7" t="s">
+      <c r="B7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E7" t="s">
+      <c r="D7" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F7"/>
-      <c r="G7" t="s">
-        <v>77</v>
-      </c>
-      <c r="H7"/>
-      <c r="I7" t="s">
+      <c r="E7" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="J7" t="b">
+      <c r="F7" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="J7" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K7"/>
-      <c r="L7" t="s">
-        <v>91</v>
-      </c>
-      <c r="M7"/>
-      <c r="N7"/>
-      <c r="O7"/>
-      <c r="P7" t="s">
+      <c r="K7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="M7" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P7" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="R7" t="s">
+      <c r="Q7" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="S7" t="s">
+      <c r="R7" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="T7" t="s">
+      <c r="S7" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="U7" t="s">
+      <c r="T7" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="V7" t="s">
+      <c r="U7" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="W7" t="s">
+      <c r="V7" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="X7" t="n">
+      <c r="W7" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="X7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="Y7"/>
-      <c r="Z7"/>
-      <c r="AA7"/>
-      <c r="AB7" t="s">
-        <v>100</v>
+      <c r="Y7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB7" s="7" t="s">
+        <v>101</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>101</v>
-      </c>
-      <c r="B8"/>
-      <c r="C8" t="s">
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D8" t="s">
+      <c r="B8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8"/>
-      <c r="G8" t="s">
-        <v>77</v>
-      </c>
-      <c r="H8"/>
-      <c r="I8" t="s">
+      <c r="D8" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="J8" t="b">
+      <c r="E8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K8"/>
-      <c r="L8" t="s">
-        <v>77</v>
-      </c>
-      <c r="M8"/>
-      <c r="N8"/>
-      <c r="O8"/>
-      <c r="P8" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>31</v>
-      </c>
-      <c r="R8" t="s">
-        <v>31</v>
-      </c>
-      <c r="S8" t="s">
-        <v>31</v>
-      </c>
-      <c r="T8" t="s">
+      <c r="K8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P8" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="U8" t="s">
+      <c r="Q8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="T8" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="V8" t="s">
+      <c r="U8" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="W8" t="s">
+      <c r="V8" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="X8" t="n">
+      <c r="W8" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="X8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="Y8"/>
-      <c r="Z8"/>
-      <c r="AA8"/>
-      <c r="AB8" t="s">
-        <v>110</v>
+      <c r="Y8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB8" s="7" t="s">
+        <v>111</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>111</v>
-      </c>
-      <c r="B9"/>
-      <c r="C9" t="s">
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D9" t="s">
+      <c r="B9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="E9" t="s">
+      <c r="D9" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F9"/>
-      <c r="G9" t="s">
+      <c r="E9" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H9"/>
-      <c r="I9" t="s">
-        <v>115</v>
-      </c>
-      <c r="J9" t="b">
+      <c r="H9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="J9" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K9"/>
-      <c r="L9" t="s">
-        <v>91</v>
-      </c>
-      <c r="M9"/>
-      <c r="N9"/>
-      <c r="O9"/>
-      <c r="P9" t="s">
+      <c r="K9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L9" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="M9" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O9" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P9" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="R9" t="s">
-        <v>116</v>
-      </c>
-      <c r="S9" t="s">
+      <c r="Q9" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="S9" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T9" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="V9" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="W9" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="X9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB9" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="J10" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N10" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P10" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q10" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R10" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T10" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="U10" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="V10" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="W10" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="X10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB10" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="J11" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L11" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N11" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O11" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q11" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="R11" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="S11" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T11" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="U11" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="V11" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="W11" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="X11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB11" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="J12" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N12" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O12" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P12" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q12" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R12" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T12" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="U12" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="V12" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="W12" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="X12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB12" s="7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="J13" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N13" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O13" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P13" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q13" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R13" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="T9" t="s">
-        <v>117</v>
-      </c>
-      <c r="U9" t="s">
+      <c r="S13" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T13" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="V13" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="W13" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="X13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB13" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="J14" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N14" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O14" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P14" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q14" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T14" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="U14" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="V14" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="W14" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="X14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z14" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA14" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB14" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="J15" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M15" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P15" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="S15" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="T15" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="V15" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="W15" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="X15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB15" s="7" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="J16" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L16" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P16" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="R16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="S16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="T16" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="U16" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="V16" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="W16" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="X16" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y16" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z16" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA16" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB16" s="7" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="J17" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L17" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N17" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O17" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P17" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q17" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="R17" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="S17" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="T17" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="U17" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="V17" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="W17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="X17" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB17" s="7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="J18" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N18" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O18" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P18" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q18" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="R18" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="S18" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="T18" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="U18" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="V18" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="W18" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="X18" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="Y18" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z18" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA18" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB18" s="7" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="J19" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L19" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="N19" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O19" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P19" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q19" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R19" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T19" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="V19" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="W19" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="X19" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z19" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA19" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB19" s="7" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="J20" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L20" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="N20" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O20" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P20" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q20" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R20" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="S20" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T20" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="U20" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="V20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="W20" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="X20" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB20" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="J21" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L21" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M21" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O21" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P21" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q21" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="S21" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T21" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="V9" t="s">
-        <v>119</v>
-      </c>
-      <c r="W9" t="s">
-        <v>120</v>
-      </c>
-      <c r="X9" t="n">
+      <c r="U21" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="V21" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="W21" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="X21" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y21" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z21" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA21" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB21" s="7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="22" ht="25" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="J22" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L22" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M22" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P22" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q22" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="R22" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="S22" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T22" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="U22" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="V22" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="W22" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="X22" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="Y9"/>
-      <c r="Z9"/>
-      <c r="AA9"/>
-      <c r="AB9" t="s">
-        <v>121</v>
+      <c r="Y22" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z22" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA22" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB22" s="7" t="s">
+        <v>252</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>122</v>
-      </c>
-      <c r="B10"/>
-      <c r="C10" t="s">
-        <v>123</v>
-      </c>
-      <c r="D10" t="s">
-        <v>124</v>
-      </c>
-      <c r="E10" t="s">
-        <v>125</v>
-      </c>
-      <c r="F10"/>
-      <c r="G10" t="s">
+    <row r="23" ht="25" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H10"/>
-      <c r="I10" t="s">
-        <v>126</v>
-      </c>
-      <c r="J10" t="b">
+      <c r="H23" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="J23" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K10"/>
-      <c r="L10" t="s">
-        <v>91</v>
-      </c>
-      <c r="M10"/>
-      <c r="N10"/>
-      <c r="O10"/>
-      <c r="P10" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>93</v>
-      </c>
-      <c r="R10" t="s">
-        <v>116</v>
-      </c>
-      <c r="S10" t="s">
-        <v>95</v>
-      </c>
-      <c r="T10" t="s">
-        <v>127</v>
-      </c>
-      <c r="U10" t="s">
-        <v>128</v>
-      </c>
-      <c r="V10" t="s">
-        <v>129</v>
-      </c>
-      <c r="W10" t="s">
-        <v>130</v>
-      </c>
-      <c r="X10" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y10"/>
-      <c r="Z10"/>
-      <c r="AA10"/>
-      <c r="AB10" t="s">
-        <v>131</v>
+      <c r="K23" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L23" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M23" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N23" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O23" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P23" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q23" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="R23" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="S23" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="T23" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="V23" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="W23" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="X23" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y23" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z23" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA23" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB23" s="7" t="s">
+        <v>263</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>132</v>
-      </c>
-      <c r="B11"/>
-      <c r="C11" t="s">
-        <v>133</v>
-      </c>
-      <c r="D11" t="s">
-        <v>134</v>
-      </c>
-      <c r="E11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11"/>
-      <c r="G11" t="s">
+    <row r="24" ht="25" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G24" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H11"/>
-      <c r="I11" t="s">
-        <v>135</v>
-      </c>
-      <c r="J11" t="b">
+      <c r="H24" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="J24" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K11"/>
-      <c r="L11" t="s">
+      <c r="K24" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L24" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M24" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N24" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O24" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P24" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q24" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="R24" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="S24" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="T24" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="U24" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="V24" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="W24" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="X24" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="Y24" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z24" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA24" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB24" s="7" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="25" ht="25" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G25" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="M11"/>
-      <c r="N11"/>
-      <c r="O11"/>
-      <c r="P11" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>136</v>
-      </c>
-      <c r="R11" t="s">
-        <v>116</v>
-      </c>
-      <c r="S11" t="s">
-        <v>95</v>
-      </c>
-      <c r="T11" t="s">
-        <v>137</v>
-      </c>
-      <c r="U11" t="s">
-        <v>138</v>
-      </c>
-      <c r="V11" t="s">
-        <v>139</v>
-      </c>
-      <c r="W11" t="s">
-        <v>140</v>
-      </c>
-      <c r="X11" t="n">
-        <v>5</v>
-      </c>
-      <c r="Y11"/>
-      <c r="Z11"/>
-      <c r="AA11"/>
-      <c r="AB11" t="s">
-        <v>141</v>
+      <c r="H25" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="J25" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L25" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M25" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N25" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O25" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P25" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q25" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="R25" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="S25" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="T25" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="U25" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="V25" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="W25" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="X25" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="Y25" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z25" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA25" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB25" s="7" t="s">
+        <v>281</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>142</v>
-      </c>
-      <c r="B12"/>
-      <c r="C12" t="s">
-        <v>143</v>
-      </c>
-      <c r="D12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E12" t="s">
-        <v>145</v>
-      </c>
-      <c r="F12"/>
-      <c r="G12" t="s">
+    <row r="26" ht="25" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H12"/>
-      <c r="I12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J12" t="b">
+      <c r="H26" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="J26" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K12"/>
-      <c r="L12" t="s">
-        <v>91</v>
-      </c>
-      <c r="M12"/>
-      <c r="N12"/>
-      <c r="O12"/>
-      <c r="P12" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>93</v>
-      </c>
-      <c r="R12" t="s">
-        <v>147</v>
-      </c>
-      <c r="S12" t="s">
-        <v>95</v>
-      </c>
-      <c r="T12" t="s">
-        <v>148</v>
-      </c>
-      <c r="U12" t="s">
-        <v>149</v>
-      </c>
-      <c r="V12" t="s">
-        <v>150</v>
-      </c>
-      <c r="W12" t="s">
-        <v>151</v>
-      </c>
-      <c r="X12" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y12"/>
-      <c r="Z12"/>
-      <c r="AA12"/>
-      <c r="AB12" t="s">
-        <v>152</v>
+      <c r="K26" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L26" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M26" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N26" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O26" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P26" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q26" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="R26" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="S26" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="T26" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="U26" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="V26" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="W26" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="X26" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y26" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z26" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA26" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB26" s="7" t="s">
+        <v>290</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>153</v>
-      </c>
-      <c r="B13"/>
-      <c r="C13" t="s">
-        <v>154</v>
-      </c>
-      <c r="D13" t="s">
-        <v>155</v>
-      </c>
-      <c r="E13" t="s">
-        <v>156</v>
-      </c>
-      <c r="F13"/>
-      <c r="G13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H13"/>
-      <c r="I13" t="s">
-        <v>157</v>
-      </c>
-      <c r="J13" t="b">
+    <row r="27" ht="25" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="J27" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K13"/>
-      <c r="L13" t="s">
-        <v>91</v>
-      </c>
-      <c r="M13"/>
-      <c r="N13"/>
-      <c r="O13"/>
-      <c r="P13" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>93</v>
-      </c>
-      <c r="R13" t="s">
-        <v>94</v>
-      </c>
-      <c r="S13" t="s">
-        <v>95</v>
-      </c>
-      <c r="T13" t="s">
-        <v>158</v>
-      </c>
-      <c r="U13" t="s">
-        <v>159</v>
-      </c>
-      <c r="V13" t="s">
-        <v>160</v>
-      </c>
-      <c r="W13" t="s">
-        <v>161</v>
-      </c>
-      <c r="X13" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y13"/>
-      <c r="Z13"/>
-      <c r="AA13"/>
-      <c r="AB13" t="s">
-        <v>162</v>
+      <c r="K27" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L27" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="M27" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N27" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O27" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P27" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q27" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="R27" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="S27" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="T27" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="U27" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="V27" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="W27" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="X27" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y27" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z27" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA27" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB27" s="7" t="s">
+        <v>299</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>163</v>
-      </c>
-      <c r="B14"/>
-      <c r="C14" t="s">
-        <v>164</v>
-      </c>
-      <c r="D14" t="s">
-        <v>165</v>
-      </c>
-      <c r="E14" t="s">
-        <v>166</v>
-      </c>
-      <c r="F14"/>
-      <c r="G14" t="s">
+    <row r="28" ht="25" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G28" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H14"/>
-      <c r="I14" t="s">
-        <v>167</v>
-      </c>
-      <c r="J14" t="b">
+      <c r="H28" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="J28" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="K14"/>
-      <c r="L14" t="s">
-        <v>91</v>
-      </c>
-      <c r="M14"/>
-      <c r="N14"/>
-      <c r="O14"/>
-      <c r="P14" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>93</v>
-      </c>
-      <c r="R14" t="s">
-        <v>147</v>
-      </c>
-      <c r="S14" t="s">
-        <v>95</v>
-      </c>
-      <c r="T14" t="s">
-        <v>168</v>
-      </c>
-      <c r="U14" t="s">
-        <v>169</v>
-      </c>
-      <c r="V14" t="s">
-        <v>170</v>
-      </c>
-      <c r="W14" t="s">
-        <v>171</v>
-      </c>
-      <c r="X14" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y14"/>
-      <c r="Z14"/>
-      <c r="AA14"/>
-      <c r="AB14" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>173</v>
-      </c>
-      <c r="B15"/>
-      <c r="C15" t="s">
-        <v>174</v>
-      </c>
-      <c r="D15" t="s">
-        <v>175</v>
-      </c>
-      <c r="E15" t="s">
-        <v>176</v>
-      </c>
-      <c r="F15"/>
-      <c r="G15" t="s">
-        <v>32</v>
-      </c>
-      <c r="H15"/>
-      <c r="I15" t="s">
-        <v>177</v>
-      </c>
-      <c r="J15" t="b">
-        <v>0</v>
-      </c>
-      <c r="K15"/>
-      <c r="L15" t="s">
-        <v>91</v>
-      </c>
-      <c r="M15"/>
-      <c r="N15"/>
-      <c r="O15"/>
-      <c r="P15" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R15" t="s">
-        <v>31</v>
-      </c>
-      <c r="S15" t="s">
-        <v>31</v>
-      </c>
-      <c r="T15" t="s">
-        <v>179</v>
-      </c>
-      <c r="U15" t="s">
-        <v>180</v>
-      </c>
-      <c r="V15" t="s">
-        <v>181</v>
-      </c>
-      <c r="W15" t="s">
-        <v>182</v>
-      </c>
-      <c r="X15" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y15"/>
-      <c r="Z15"/>
-      <c r="AA15"/>
-      <c r="AB15" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>184</v>
-      </c>
-      <c r="B16"/>
-      <c r="C16" t="s">
-        <v>185</v>
-      </c>
-      <c r="D16" t="s">
-        <v>186</v>
-      </c>
-      <c r="E16" t="s">
-        <v>187</v>
-      </c>
-      <c r="F16"/>
-      <c r="G16" t="s">
-        <v>32</v>
-      </c>
-      <c r="H16"/>
-      <c r="I16" t="s">
-        <v>188</v>
-      </c>
-      <c r="J16" t="b">
-        <v>0</v>
-      </c>
-      <c r="K16"/>
-      <c r="L16" t="s">
-        <v>91</v>
-      </c>
-      <c r="M16"/>
-      <c r="N16"/>
-      <c r="O16"/>
-      <c r="P16" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>31</v>
-      </c>
-      <c r="R16" t="s">
-        <v>31</v>
-      </c>
-      <c r="S16" t="s">
-        <v>31</v>
-      </c>
-      <c r="T16" t="s">
-        <v>189</v>
-      </c>
-      <c r="U16" t="s">
-        <v>190</v>
-      </c>
-      <c r="V16" t="s">
-        <v>191</v>
-      </c>
-      <c r="W16" t="s">
-        <v>192</v>
-      </c>
-      <c r="X16" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y16"/>
-      <c r="Z16"/>
-      <c r="AA16"/>
-      <c r="AB16" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>194</v>
-      </c>
-      <c r="B17"/>
-      <c r="C17" t="s">
-        <v>195</v>
-      </c>
-      <c r="D17" t="s">
-        <v>196</v>
-      </c>
-      <c r="E17" t="s">
-        <v>31</v>
-      </c>
-      <c r="F17"/>
-      <c r="G17" t="s">
-        <v>77</v>
-      </c>
-      <c r="H17"/>
-      <c r="I17" t="s">
-        <v>197</v>
-      </c>
-      <c r="J17" t="b">
-        <v>0</v>
-      </c>
-      <c r="K17"/>
-      <c r="L17" t="s">
-        <v>77</v>
-      </c>
-      <c r="M17"/>
-      <c r="N17"/>
-      <c r="O17"/>
-      <c r="P17" t="s">
+      <c r="K28" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L28" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="Q17" t="s">
-        <v>80</v>
-      </c>
-      <c r="R17" t="s">
-        <v>198</v>
-      </c>
-      <c r="S17" t="s">
-        <v>37</v>
-      </c>
-      <c r="T17" t="s">
-        <v>199</v>
-      </c>
-      <c r="U17" t="s">
-        <v>200</v>
-      </c>
-      <c r="V17" t="s">
-        <v>201</v>
-      </c>
-      <c r="W17" t="s">
-        <v>31</v>
-      </c>
-      <c r="X17" t="n">
-        <v>5</v>
-      </c>
-      <c r="Y17"/>
-      <c r="Z17"/>
-      <c r="AA17"/>
-      <c r="AB17" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>203</v>
-      </c>
-      <c r="B18"/>
-      <c r="C18" t="s">
-        <v>204</v>
-      </c>
-      <c r="D18" t="s">
-        <v>205</v>
-      </c>
-      <c r="E18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18"/>
-      <c r="G18" t="s">
-        <v>77</v>
-      </c>
-      <c r="H18"/>
-      <c r="I18" t="s">
-        <v>206</v>
-      </c>
-      <c r="J18" t="b">
-        <v>0</v>
-      </c>
-      <c r="K18"/>
-      <c r="L18" t="s">
-        <v>77</v>
-      </c>
-      <c r="M18"/>
-      <c r="N18"/>
-      <c r="O18"/>
-      <c r="P18" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>31</v>
-      </c>
-      <c r="R18" t="s">
-        <v>31</v>
-      </c>
-      <c r="S18" t="s">
-        <v>31</v>
-      </c>
-      <c r="T18" t="s">
-        <v>207</v>
-      </c>
-      <c r="U18" t="s">
-        <v>208</v>
-      </c>
-      <c r="V18" t="s">
-        <v>209</v>
-      </c>
-      <c r="W18" t="s">
-        <v>210</v>
-      </c>
-      <c r="X18" t="n">
-        <v>11</v>
-      </c>
-      <c r="Y18"/>
-      <c r="Z18"/>
-      <c r="AA18"/>
-      <c r="AB18" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>212</v>
-      </c>
-      <c r="B19"/>
-      <c r="C19" t="s">
-        <v>213</v>
-      </c>
-      <c r="D19" t="s">
-        <v>214</v>
-      </c>
-      <c r="E19" t="s">
-        <v>215</v>
-      </c>
-      <c r="F19"/>
-      <c r="G19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H19"/>
-      <c r="I19" t="s">
-        <v>216</v>
-      </c>
-      <c r="J19" t="b">
-        <v>0</v>
-      </c>
-      <c r="K19"/>
-      <c r="L19" t="s">
-        <v>91</v>
-      </c>
-      <c r="M19"/>
-      <c r="N19"/>
-      <c r="O19"/>
-      <c r="P19" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>93</v>
-      </c>
-      <c r="R19" t="s">
-        <v>217</v>
-      </c>
-      <c r="S19" t="s">
-        <v>95</v>
-      </c>
-      <c r="T19" t="s">
-        <v>218</v>
-      </c>
-      <c r="U19" t="s">
-        <v>219</v>
-      </c>
-      <c r="V19" t="s">
-        <v>220</v>
-      </c>
-      <c r="W19" t="s">
-        <v>221</v>
-      </c>
-      <c r="X19" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y19"/>
-      <c r="Z19"/>
-      <c r="AA19"/>
-      <c r="AB19" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>223</v>
-      </c>
-      <c r="B20"/>
-      <c r="C20" t="s">
-        <v>224</v>
-      </c>
-      <c r="D20" t="s">
-        <v>225</v>
-      </c>
-      <c r="E20" t="s">
-        <v>226</v>
-      </c>
-      <c r="F20"/>
-      <c r="G20" t="s">
-        <v>77</v>
-      </c>
-      <c r="H20"/>
-      <c r="I20" t="s">
-        <v>227</v>
-      </c>
-      <c r="J20" t="b">
-        <v>0</v>
-      </c>
-      <c r="K20"/>
-      <c r="L20" t="s">
-        <v>91</v>
-      </c>
-      <c r="M20"/>
-      <c r="N20"/>
-      <c r="O20"/>
-      <c r="P20" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>93</v>
-      </c>
-      <c r="R20" t="s">
-        <v>217</v>
-      </c>
-      <c r="S20" t="s">
-        <v>95</v>
-      </c>
-      <c r="T20" t="s">
-        <v>228</v>
-      </c>
-      <c r="U20" t="s">
-        <v>229</v>
-      </c>
-      <c r="V20" t="s">
-        <v>230</v>
-      </c>
-      <c r="W20" t="s">
-        <v>231</v>
-      </c>
-      <c r="X20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y20"/>
-      <c r="Z20"/>
-      <c r="AA20"/>
-      <c r="AB20" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>233</v>
-      </c>
-      <c r="B21"/>
-      <c r="C21" t="s">
-        <v>234</v>
-      </c>
-      <c r="D21" t="s">
-        <v>235</v>
-      </c>
-      <c r="E21" t="s">
-        <v>236</v>
-      </c>
-      <c r="F21"/>
-      <c r="G21" t="s">
-        <v>77</v>
-      </c>
-      <c r="H21"/>
-      <c r="I21" t="s">
-        <v>237</v>
-      </c>
-      <c r="J21" t="b">
-        <v>0</v>
-      </c>
-      <c r="K21"/>
-      <c r="L21" t="s">
-        <v>91</v>
-      </c>
-      <c r="M21"/>
-      <c r="N21"/>
-      <c r="O21"/>
-      <c r="P21" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>93</v>
-      </c>
-      <c r="R21" t="s">
-        <v>217</v>
-      </c>
-      <c r="S21" t="s">
-        <v>95</v>
-      </c>
-      <c r="T21" t="s">
-        <v>117</v>
-      </c>
-      <c r="U21" t="s">
-        <v>238</v>
-      </c>
-      <c r="V21" t="s">
-        <v>239</v>
-      </c>
-      <c r="W21" t="s">
-        <v>240</v>
-      </c>
-      <c r="X21" t="n">
-        <v>5</v>
-      </c>
-      <c r="Y21"/>
-      <c r="Z21"/>
-      <c r="AA21"/>
-      <c r="AB21" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>242</v>
-      </c>
-      <c r="B22"/>
-      <c r="C22" t="s">
-        <v>243</v>
-      </c>
-      <c r="D22" t="s">
-        <v>244</v>
-      </c>
-      <c r="E22" t="s">
-        <v>245</v>
-      </c>
-      <c r="F22"/>
-      <c r="G22" t="s">
-        <v>77</v>
-      </c>
-      <c r="H22"/>
-      <c r="I22" t="s">
-        <v>246</v>
-      </c>
-      <c r="J22" t="b">
-        <v>0</v>
-      </c>
-      <c r="K22"/>
-      <c r="L22" t="s">
-        <v>91</v>
-      </c>
-      <c r="M22"/>
-      <c r="N22"/>
-      <c r="O22"/>
-      <c r="P22" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>247</v>
-      </c>
-      <c r="R22" t="s">
-        <v>248</v>
-      </c>
-      <c r="S22" t="s">
-        <v>95</v>
-      </c>
-      <c r="T22" t="s">
-        <v>117</v>
-      </c>
-      <c r="U22" t="s">
-        <v>249</v>
-      </c>
-      <c r="V22" t="s">
-        <v>250</v>
-      </c>
-      <c r="W22" t="s">
-        <v>251</v>
-      </c>
-      <c r="X22" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y22"/>
-      <c r="Z22"/>
-      <c r="AA22"/>
-      <c r="AB22" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>253</v>
-      </c>
-      <c r="B23"/>
-      <c r="C23" t="s">
-        <v>254</v>
-      </c>
-      <c r="D23" t="s">
-        <v>255</v>
-      </c>
-      <c r="E23" t="s">
-        <v>31</v>
-      </c>
-      <c r="F23"/>
-      <c r="G23" t="s">
-        <v>77</v>
-      </c>
-      <c r="H23"/>
-      <c r="I23" t="s">
-        <v>256</v>
-      </c>
-      <c r="J23" t="b">
-        <v>0</v>
-      </c>
-      <c r="K23"/>
-      <c r="L23" t="s">
-        <v>77</v>
-      </c>
-      <c r="M23"/>
-      <c r="N23"/>
-      <c r="O23"/>
-      <c r="P23" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q23" t="s">
+      <c r="M28" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N28" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O28" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P28" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q28" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="R23" t="s">
+      <c r="R28" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="S23" t="s">
+      <c r="S28" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="T23" t="s">
-        <v>259</v>
-      </c>
-      <c r="U23" t="s">
-        <v>260</v>
-      </c>
-      <c r="V23" t="s">
-        <v>261</v>
-      </c>
-      <c r="W23" t="s">
-        <v>262</v>
-      </c>
-      <c r="X23" t="n">
+      <c r="T28" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="U28" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="V28" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="W28" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="X28" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="Y23"/>
-      <c r="Z23"/>
-      <c r="AA23"/>
-      <c r="AB23" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>264</v>
-      </c>
-      <c r="B24"/>
-      <c r="C24" t="s">
-        <v>265</v>
-      </c>
-      <c r="D24" t="s">
-        <v>266</v>
-      </c>
-      <c r="E24" t="s">
-        <v>31</v>
-      </c>
-      <c r="F24"/>
-      <c r="G24" t="s">
-        <v>77</v>
-      </c>
-      <c r="H24"/>
-      <c r="I24" t="s">
-        <v>267</v>
-      </c>
-      <c r="J24" t="b">
-        <v>0</v>
-      </c>
-      <c r="K24"/>
-      <c r="L24" t="s">
-        <v>77</v>
-      </c>
-      <c r="M24"/>
-      <c r="N24"/>
-      <c r="O24"/>
-      <c r="P24" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>257</v>
-      </c>
-      <c r="R24" t="s">
-        <v>258</v>
-      </c>
-      <c r="S24" t="s">
-        <v>258</v>
-      </c>
-      <c r="T24" t="s">
-        <v>268</v>
-      </c>
-      <c r="U24" t="s">
-        <v>269</v>
-      </c>
-      <c r="V24" t="s">
-        <v>270</v>
-      </c>
-      <c r="W24" t="s">
-        <v>271</v>
-      </c>
-      <c r="X24" t="n">
-        <v>11</v>
-      </c>
-      <c r="Y24"/>
-      <c r="Z24"/>
-      <c r="AA24"/>
-      <c r="AB24" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>273</v>
-      </c>
-      <c r="B25"/>
-      <c r="C25" t="s">
-        <v>274</v>
-      </c>
-      <c r="D25" t="s">
-        <v>275</v>
-      </c>
-      <c r="E25" t="s">
-        <v>31</v>
-      </c>
-      <c r="F25"/>
-      <c r="G25" t="s">
-        <v>77</v>
-      </c>
-      <c r="H25"/>
-      <c r="I25" t="s">
-        <v>276</v>
-      </c>
-      <c r="J25" t="b">
-        <v>0</v>
-      </c>
-      <c r="K25"/>
-      <c r="L25" t="s">
-        <v>77</v>
-      </c>
-      <c r="M25"/>
-      <c r="N25"/>
-      <c r="O25"/>
-      <c r="P25" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>257</v>
-      </c>
-      <c r="R25" t="s">
-        <v>258</v>
-      </c>
-      <c r="S25" t="s">
-        <v>258</v>
-      </c>
-      <c r="T25" t="s">
-        <v>277</v>
-      </c>
-      <c r="U25" t="s">
-        <v>278</v>
-      </c>
-      <c r="V25" t="s">
-        <v>279</v>
-      </c>
-      <c r="W25" t="s">
-        <v>280</v>
-      </c>
-      <c r="X25" t="n">
-        <v>11</v>
-      </c>
-      <c r="Y25"/>
-      <c r="Z25"/>
-      <c r="AA25"/>
-      <c r="AB25" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>282</v>
-      </c>
-      <c r="B26"/>
-      <c r="C26" t="s">
-        <v>283</v>
-      </c>
-      <c r="D26" t="s">
-        <v>284</v>
-      </c>
-      <c r="E26" t="s">
-        <v>31</v>
-      </c>
-      <c r="F26"/>
-      <c r="G26" t="s">
-        <v>77</v>
-      </c>
-      <c r="H26"/>
-      <c r="I26" t="s">
-        <v>285</v>
-      </c>
-      <c r="J26" t="b">
-        <v>0</v>
-      </c>
-      <c r="K26"/>
-      <c r="L26" t="s">
-        <v>77</v>
-      </c>
-      <c r="M26"/>
-      <c r="N26"/>
-      <c r="O26"/>
-      <c r="P26" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>257</v>
-      </c>
-      <c r="R26" t="s">
-        <v>258</v>
-      </c>
-      <c r="S26" t="s">
-        <v>258</v>
-      </c>
-      <c r="T26" t="s">
-        <v>286</v>
-      </c>
-      <c r="U26" t="s">
-        <v>287</v>
-      </c>
-      <c r="V26" t="s">
-        <v>288</v>
-      </c>
-      <c r="W26" t="s">
-        <v>289</v>
-      </c>
-      <c r="X26" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y26"/>
-      <c r="Z26"/>
-      <c r="AA26"/>
-      <c r="AB26" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s">
-        <v>291</v>
-      </c>
-      <c r="B27"/>
-      <c r="C27" t="s">
-        <v>292</v>
-      </c>
-      <c r="D27" t="s">
-        <v>293</v>
-      </c>
-      <c r="E27" t="s">
-        <v>31</v>
-      </c>
-      <c r="F27"/>
-      <c r="G27" t="s">
-        <v>77</v>
-      </c>
-      <c r="H27"/>
-      <c r="I27" t="s">
-        <v>294</v>
-      </c>
-      <c r="J27" t="b">
-        <v>0</v>
-      </c>
-      <c r="K27"/>
-      <c r="L27" t="s">
-        <v>77</v>
-      </c>
-      <c r="M27"/>
-      <c r="N27"/>
-      <c r="O27"/>
-      <c r="P27" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q27" t="s">
-        <v>257</v>
-      </c>
-      <c r="R27" t="s">
-        <v>258</v>
-      </c>
-      <c r="S27" t="s">
-        <v>258</v>
-      </c>
-      <c r="T27" t="s">
-        <v>295</v>
-      </c>
-      <c r="U27" t="s">
-        <v>296</v>
-      </c>
-      <c r="V27" t="s">
-        <v>297</v>
-      </c>
-      <c r="W27" t="s">
-        <v>298</v>
-      </c>
-      <c r="X27" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y27"/>
-      <c r="Z27"/>
-      <c r="AA27"/>
-      <c r="AB27" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s">
-        <v>300</v>
-      </c>
-      <c r="B28"/>
-      <c r="C28" t="s">
-        <v>301</v>
-      </c>
-      <c r="D28" t="s">
-        <v>302</v>
-      </c>
-      <c r="E28" t="s">
-        <v>31</v>
-      </c>
-      <c r="F28"/>
-      <c r="G28" t="s">
-        <v>77</v>
-      </c>
-      <c r="H28"/>
-      <c r="I28" t="s">
-        <v>303</v>
-      </c>
-      <c r="J28" t="b">
-        <v>0</v>
-      </c>
-      <c r="K28"/>
-      <c r="L28" t="s">
-        <v>77</v>
-      </c>
-      <c r="M28"/>
-      <c r="N28"/>
-      <c r="O28"/>
-      <c r="P28" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>257</v>
-      </c>
-      <c r="R28" t="s">
-        <v>258</v>
-      </c>
-      <c r="S28" t="s">
-        <v>258</v>
-      </c>
-      <c r="T28" t="s">
-        <v>304</v>
-      </c>
-      <c r="U28" t="s">
-        <v>305</v>
-      </c>
-      <c r="V28" t="s">
-        <v>306</v>
-      </c>
-      <c r="W28" t="s">
-        <v>307</v>
-      </c>
-      <c r="X28" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y28"/>
-      <c r="Z28"/>
-      <c r="AA28"/>
-      <c r="AB28" t="s">
+      <c r="Y28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB28" s="7" t="s">
         <v>308</v>
       </c>
     </row>

</xml_diff>